<commit_message>
Reconcile transport plan: no rental beyond Florence-Tuscany, drop Pompeii
Origin had already reordered Naples before Amalfi independently but kept
self-driving the whole coast and FCO-to-FCO, and priced Naples at a
guessed $1,098. This corrects it to match the confirmed De Bonart
booking ($1,071) and the actual plan: rental car returns to Florence
Sep 1 (the Florence->Naples train doesn't run from Castelfalfi),
private drivers cover both Naples<->Amalfi legs, rail covers
Naples->Rome, and Pompeii is dropped since there's no car to route
through it with. Keeps origin's more precise Rome/Tuscany hotel quotes,
CLAUDE.md, and mobile CSS fixes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/italy-2026/dist/Italy 2026 (revised).xlsx
+++ b/italy-2026/dist/Italy 2026 (revised).xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="463">
   <si>
     <t>ITALY 2026 PLAN</t>
   </si>
@@ -58,7 +58,7 @@
     <t>Transport</t>
   </si>
   <si>
-    <t>Private driver in from FCO · Frecciarossa to Florence · self-drive from Aug 29 (Florence → FCO), IDP in hand</t>
+    <t>Private driver in from FCO · Frecciarossa to Florence · self-drive Florence–Tuscany only (Aug 29 – Sep 1) · rail + private drivers from Naples on, IDP in hand</t>
   </si>
   <si>
     <t>Chain story</t>
@@ -655,133 +655,124 @@
     <t>Tue, Sep 1</t>
   </si>
   <si>
-    <t>TUSCANY → NAPLES — De Bonart</t>
-  </si>
-  <si>
-    <t>Watch this: The longest drive of the trip — roughly five hours of autostrada, most of it past Rome and Caserta. Fill the tank before you leave Castelfalfi, swap drivers if you can, and expect Naples traffic to eat the last half hour.</t>
-  </si>
-  <si>
-    <t>8:00am</t>
-  </si>
-  <si>
-    <t>Check out; on the road — South on the A1 — Florence's ring road, then the long autostrada stretch past Rome and Caserta</t>
-  </si>
-  <si>
-    <t>10:45am</t>
-  </si>
-  <si>
-    <t>Fuel and coffee stop — An Autogrill service area north of Rome — top up the tank, swap drivers</t>
-  </si>
-  <si>
-    <t>Check in — De Bonart, Curio Collection — An art palazzo on Via Partenope in Chiaia, facing the bay. Hand the car to the hotel valet and leave it there — you won't need it again until Thursday.</t>
-  </si>
-  <si>
-    <t>Naples Archaeological Museum — The frescoes, mosaics and bronzes lifted out of Pompeii all ended up here. You see the rooms they came from on Thursday, so this is the right way round.</t>
+    <t>TUSCANY → NAPLES — return the car in Florence, then the train</t>
+  </si>
+  <si>
+    <t>8:30am</t>
+  </si>
+  <si>
+    <t>Check out; drive to Florence — Back the way you came — about ninety minutes, less traffic than the Friday-afternoon drive in</t>
+  </si>
+  <si>
+    <t>Drop off the rental car — Borgo Ognissanti, near Firenze S.M.N. — reservation #21586310US4 ends here</t>
+  </si>
+  <si>
+    <t>Rental desk</t>
+  </si>
+  <si>
+    <t>Coffee, then the platform — A buffer before the train — Frecciarossa 9413 doesn't wait</t>
+  </si>
+  <si>
+    <t>12:48pm</t>
+  </si>
+  <si>
+    <t>Frecciarossa 9413 to Naples — Firenze S.M.N. → Napoli Centrale, direct — 3h15. Super Economy fare, from €71.80.</t>
+  </si>
+  <si>
+    <t>Train</t>
+  </si>
+  <si>
+    <t>4:03pm</t>
+  </si>
+  <si>
+    <t>Arrive Napoli Centrale</t>
+  </si>
+  <si>
+    <t>4:30pm</t>
+  </si>
+  <si>
+    <t>Check in — De Bonart, Curio Collection — An art palazzo on Via Partenope in Chiaia, facing the bay</t>
+  </si>
+  <si>
+    <t>Rooftop aperitivo — Vesuvius on one side, the bay on the other</t>
+  </si>
+  <si>
+    <t>Dinner — pizza at Sorbillo — Via dei Tribunali. You are in the city that invented it; do this before anything fancier.</t>
+  </si>
+  <si>
+    <t>Wed, Sep 2</t>
+  </si>
+  <si>
+    <t>NAPLES — Capri day trip</t>
+  </si>
+  <si>
+    <t>Walk down to Molo Beverello — The fast-ferry pier is fifteen minutes along the seafront from the hotel</t>
+  </si>
+  <si>
+    <t>Walk, ~15 min</t>
+  </si>
+  <si>
+    <t>9:20am</t>
+  </si>
+  <si>
+    <t>Fast ferry — Naples → Capri — NLG, SNAV and Caremar all run it in about fifty minutes. Sailings are frequent in September but sell out at the counter — book online the night before.</t>
+  </si>
+  <si>
+    <t>Fast ferry, ~50 min</t>
+  </si>
+  <si>
+    <t>Timetable -&gt;</t>
+  </si>
+  <si>
+    <t>The Faraglioni, the grottoes, the swim coves — Pick up a round-the-island boat at Marina Grande — Blue Grotto if the sea is calm enough to enter</t>
+  </si>
+  <si>
+    <t>Local boat from Marina Grande</t>
+  </si>
+  <si>
+    <t>Lunch — Da Paolino — Under the lemon trees. Il Riccio is the Michelin alternative, on the cliff by the grotto.</t>
+  </si>
+  <si>
+    <t>Marina Grande, then the funicular</t>
+  </si>
+  <si>
+    <t>The Piazzetta and the Gardens of Augustus — Gelato on the terrace above Via Krupp</t>
+  </si>
+  <si>
+    <t>6:15pm</t>
+  </si>
+  <si>
+    <t>Ferry back to Naples — Check the final sailing when you arrive — the last fast boats go early evening, and missing one means a night on the island</t>
+  </si>
+  <si>
+    <t>Dinner — Palazzo Petrucci — Michelin-starred Neapolitan tasting menu, back in the old city — the celebration dinner for the boat day</t>
+  </si>
+  <si>
+    <t>Thu, Sep 3</t>
+  </si>
+  <si>
+    <t>NAPLES → AMALFI — private driver</t>
+  </si>
+  <si>
+    <t>Pizza for breakfast — Di Matteo — Also on Via dei Tribunali, a few doors from last night's Sorbillo. Yes, at 8:30am. It's Naples.</t>
   </si>
   <si>
     <t>Spaccanapoli — The dead-straight Greek road that still splits the old city in half</t>
   </si>
   <si>
-    <t>Walk from the museum</t>
-  </si>
-  <si>
-    <t>Street food, standing up — Pizza fritta, zeppoline, a sfogliatella riccia straight from the oven</t>
-  </si>
-  <si>
-    <t>Rooftop aperitivo — Vesuvius on one side, the bay on the other</t>
-  </si>
-  <si>
-    <t>9:15pm</t>
-  </si>
-  <si>
-    <t>Dinner — pizza on Via dei Tribunali — Sorbillo or Di Matteo. You are in the city that invented it; do this before anything fancier.</t>
-  </si>
-  <si>
-    <t>Wed, Sep 2</t>
-  </si>
-  <si>
-    <t>NAPLES — Capri day trip</t>
-  </si>
-  <si>
-    <t>8:30am</t>
-  </si>
-  <si>
-    <t>Walk down to Molo Beverello — The fast-ferry pier is fifteen minutes along the seafront from the hotel</t>
-  </si>
-  <si>
-    <t>Walk, ~15 min</t>
-  </si>
-  <si>
-    <t>9:20am</t>
-  </si>
-  <si>
-    <t>Fast ferry — Naples → Capri — NLG, SNAV and Caremar all run it in about fifty minutes. Sailings are frequent in September but sell out at the counter — book online the night before.</t>
-  </si>
-  <si>
-    <t>Fast ferry, ~50 min</t>
-  </si>
-  <si>
-    <t>Timetable -&gt;</t>
-  </si>
-  <si>
-    <t>The Faraglioni, the grottoes, the swim coves — Pick up a round-the-island boat at Marina Grande — Blue Grotto if the sea is calm enough to enter</t>
-  </si>
-  <si>
-    <t>Local boat from Marina Grande</t>
-  </si>
-  <si>
-    <t>Lunch — Da Paolino — Under the lemon trees. Il Riccio is the Michelin alternative, on the cliff by the grotto.</t>
-  </si>
-  <si>
-    <t>Marina Grande, then the funicular</t>
-  </si>
-  <si>
-    <t>The Piazzetta and the Gardens of Augustus — Gelato on the terrace above Via Krupp</t>
-  </si>
-  <si>
-    <t>6:15pm</t>
-  </si>
-  <si>
-    <t>Ferry back to Naples — Check the final sailing when you arrive — the last fast boats go early evening, and missing one means a night on the island</t>
-  </si>
-  <si>
-    <t>Dinner — Palazzo Petrucci — Michelin-starred Neapolitan tasting menu, back in the old city</t>
-  </si>
-  <si>
-    <t>Thu, Sep 3</t>
-  </si>
-  <si>
-    <t>NAPLES → AMALFI, via Pompeii</t>
-  </si>
-  <si>
-    <t>Check out; collect the car from the valet — First time behind the wheel since Tuesday</t>
-  </si>
-  <si>
-    <t>9:15am</t>
-  </si>
-  <si>
-    <t>Drive to Pompeii — Half an hour southeast on the A3 — exit for Pompei Scavi</t>
-  </si>
-  <si>
-    <t>Self-drive, ~30 min</t>
-  </si>
-  <si>
-    <t>Pompeii, guided — Two and a half hours is the right length in September heat. Ask for the Villa of the Mysteries. Parking is at the Pompei Scavi lot by the entrance.</t>
-  </si>
-  <si>
-    <t>Arrive; on-site parking</t>
-  </si>
-  <si>
-    <t>Lunch, then onto the corniche — The coast road starts properly after Vietri — narrow, slow, spectacular. Take it easy.</t>
+    <t>Check out; last look at the bay</t>
+  </si>
+  <si>
+    <t>Private driver to Amalfi — Coast road via Vietri — narrow, slow, spectacular. Sit back, someone else is driving.</t>
+  </si>
+  <si>
+    <t>Private driver, ~1.5–2 hrs</t>
   </si>
   <si>
     <t>Check in — Anantara Convento di Amalfi — A 13th-century monastery on the cliff edge, with the original cloister still standing</t>
   </si>
   <si>
-    <t>Scenic drive, ~1.5 hrs</t>
-  </si>
-  <si>
-    <t>The beach club, by cliff lift — Down to sea level for what's left of the afternoon</t>
+    <t>The beach club, by cliff lift — A slow afternoon at sea level after the drive</t>
   </si>
   <si>
     <t>Hotel cliff lift</t>
@@ -814,6 +805,9 @@
     <t>Up to Ravello — Forty-five minutes of switchbacks above the coast</t>
   </si>
   <si>
+    <t>Private driver</t>
+  </si>
+  <si>
     <t>3:45pm</t>
   </si>
   <si>
@@ -847,13 +841,25 @@
     <t>Sat, Sep 5</t>
   </si>
   <si>
-    <t>AMALFI → ROME — The St. Regis</t>
-  </si>
-  <si>
-    <t>Check out; last look at the coast — Breakfast on the cloister terrace before you give the cliff back</t>
-  </si>
-  <si>
-    <t>Down the corniche, then north — The coast road as far as Vietri, then the A3 and the A1 — Amalfi → Rome is about four hours all told</t>
+    <t>AMALFI → NAPLES → ROME — driver, then train</t>
+  </si>
+  <si>
+    <t>Check out; last look at the coast — Breakfast on the cloister terrace before you give the room back</t>
+  </si>
+  <si>
+    <t>Private driver to Naples — Back along the coast road to Napoli Centrale</t>
+  </si>
+  <si>
+    <t>Private driver, ~1.5 hrs</t>
+  </si>
+  <si>
+    <t>Arrive Napoli Centrale; drop bags, coffee</t>
+  </si>
+  <si>
+    <t>Frecciarossa to Rome — Napoli Centrale → Roma Termini, direct — about 1h10. Frequent departures; no need to book far ahead.</t>
+  </si>
+  <si>
+    <t>Arrive Roma Termini; taxi to the hotel</t>
   </si>
   <si>
     <t>Check in — The St. Regis Rome — The hotel is inside Rome's ZTL — use valet or a garage nearby; don't try to park at the curb.</t>
@@ -874,13 +880,10 @@
     <t>DEPART — FCO → IAH</t>
   </si>
   <si>
-    <t>Watch this: The rental is booked for a 12:00pm drop-off, but the flight leaves at 10:20am — the car would still be at FCO after you've taken off. Call the rental company and move the drop-off to around 6:00am.</t>
-  </si>
-  <si>
-    <t>6:00am</t>
-  </si>
-  <si>
-    <t>Drive to FCO; drop off the car — About forty minutes on an empty Sunday road — reservation #21586310US4</t>
+    <t>6:40am</t>
+  </si>
+  <si>
+    <t>Taxi to FCO — About forty minutes on an empty Sunday road. No rental to return this time — that ended in Florence on Sep 1.</t>
   </si>
   <si>
     <t>7:20am</t>
@@ -997,16 +1000,16 @@
     <t>Lodging</t>
   </si>
   <si>
-    <t>6 hotels, 13 nights. Trame ($1,571.58), Castelfalfi ($3,764.98) and De Bonart ($1,098.27) are confirmed bookings; Convento is a quote, now 2 nights rather than 3. The St. Regis is still an estimate.</t>
-  </si>
-  <si>
-    <t>Holding the old total pending a re-quote: the rental drops from 14 days to 8 (Florence Aug 29 → FCO Sep 6), but a one-way pickup fee eats into that, and the FCO private transfer (~€70–90) and two Frecciarossa fares are new. Rome garage parking is gone entirely. Fuel and tolls now only from Aug 29.</t>
+    <t>6 hotels, 13 nights. Trame ($1,571.58), Castelfalfi ($3,764.98) and De Bonart ($1,071, confirmed) are actual bookings; Convento is a quote, 2 nights rather than 3. The St. Regis is still an estimate.</t>
+  </si>
+  <si>
+    <t>Holding the old total pending a re-quote: the rental drops from 14 days to 3 (Florence Aug 29 → Florence Sep 1, both ends the same city now), but a one-way-turned-round-trip re-quote could move that either way. New costs: the FCO private transfer (~€70–90), two Frecciarossa fares, and private drivers for both Naples↔Amalfi legs. Rome and FCO parking are gone entirely.</t>
   </si>
   <si>
     <t>Excursions &amp; guides</t>
   </si>
   <si>
-    <t>Vatican, Colosseum, Pompeii, Capri, wineries, Florence galleries, operas. Held pending a re-quote: swapping the private Lucibello charter for the Capri ferry takes a four-figure line down to about €50 of tickets for the two of you, so this should come down materially.</t>
+    <t>Vatican, Colosseum, Capri, wineries, Florence galleries, operas. Held pending a re-quote: swapping the private Lucibello charter for the Capri ferry takes a four-figure line down to about €50 of tickets for the two of you, and dropping Pompeii removes a guide fee, so this should come down materially.</t>
   </si>
   <si>
     <t>Food &amp; wine</t>
@@ -1036,9 +1039,6 @@
     <t>Aug 24</t>
   </si>
   <si>
-    <t>Private driver</t>
-  </si>
-  <si>
     <t>FCO → Hotel Trame, Rome  (Pre-booked NCC, name board at arrivals — book before you fly)</t>
   </si>
   <si>
@@ -1105,61 +1105,70 @@
     <t>Sep 1</t>
   </si>
   <si>
-    <t>Il Castelfalfi → De Bonart Naples  (The longest drive of the trip — then the car goes to the hotel valet until Thursday)</t>
+    <t>Self-drive, then train</t>
+  </si>
+  <si>
+    <t>Il Castelfalfi → Firenze S.M.N. (drop the car) → Napoli Centrale  (Frecciarossa 9413, 12:48 → 16:03. Return the rental in Florence before the train — it does not go on to Naples.)</t>
+  </si>
+  <si>
+    <t>~1.5 hrs drive + 3h15 train</t>
+  </si>
+  <si>
+    <t>Sep 2</t>
+  </si>
+  <si>
+    <t>Fast ferry</t>
+  </si>
+  <si>
+    <t>Molo Beverello, Naples → Capri → back  (NLG / SNAV / Caremar — book online the night before, and check the last sailing back)</t>
+  </si>
+  <si>
+    <t>~50 min each way</t>
+  </si>
+  <si>
+    <t>Sep 3</t>
+  </si>
+  <si>
+    <t>De Bonart Naples → Anantara Convento, Amalfi  (No rental car for this leg, and Pompeii is dropped with it — book a car service for the coast road)</t>
+  </si>
+  <si>
+    <t>~1.5–2 hrs</t>
+  </si>
+  <si>
+    <t>Sep 4</t>
+  </si>
+  <si>
+    <t>Anantara Convento → Ravello (evening concert) → back  (Tight switchbacks, and no rental car by this point — a local driver is the only option, not just the easy one)</t>
   </si>
   <si>
     <t>~5 hrs</t>
   </si>
   <si>
-    <t>Sep 2</t>
-  </si>
-  <si>
-    <t>Fast ferry</t>
-  </si>
-  <si>
-    <t>Molo Beverello, Naples → Capri → back  (NLG / SNAV / Caremar — book online the night before, and check the last sailing back)</t>
-  </si>
-  <si>
-    <t>~50 min each way</t>
-  </si>
-  <si>
-    <t>Sep 3</t>
-  </si>
-  <si>
-    <t>Naples → Pompeii (guided) → Anantara Convento, Amalfi  (Pompeii is directly on the way — no detour at all)</t>
-  </si>
-  <si>
-    <t>~5 hrs with the site</t>
-  </si>
-  <si>
-    <t>Sep 4</t>
-  </si>
-  <si>
-    <t>Anantara Convento → Ravello (evening concert) → back  (Tight switchbacks — a local driver is a fine substitute for this one leg)</t>
-  </si>
-  <si>
     <t>Sep 5</t>
   </si>
   <si>
-    <t>Anantara Convento → The St. Regis Rome  (Corniche as far as Vietri, then the A3 and A1)</t>
-  </si>
-  <si>
-    <t>~4 hrs</t>
+    <t>Anantara Convento, Amalfi → Napoli Centrale</t>
+  </si>
+  <si>
+    <t>~1.5 hrs</t>
+  </si>
+  <si>
+    <t>Napoli Centrale → Roma Termini (Frecciarossa)  (Frequent departures — no need to pre-book far ahead)</t>
+  </si>
+  <si>
+    <t>~1h10</t>
   </si>
   <si>
     <t>Sep 6</t>
   </si>
   <si>
-    <t>Drop off the car</t>
-  </si>
-  <si>
-    <t>The St. Regis Rome → FCO  (Drop-off is booked for noon — move it earlier so it isn't after the flight)</t>
+    <t>The St. Regis Rome → FCO  (No rental to return — that was dropped off in Florence on Sep 1)</t>
   </si>
   <si>
     <t>~40 min</t>
   </si>
   <si>
-    <t>You are car-free for the first five days: a private driver in from FCO, taxis and your feet in Rome, the Frecciarossa to Florence. The car is only collected on Aug 29, on Borgo Ognissanti just outside Florence's ZTL, and runs from there to the FCO drop-off on Sep 6 — eight days rather than fourteen, and no Rome garage at all. The IDP ships by Aug 3; pack it with the physical licence, not just a photo of it. Never drive into either historic centre — Florence's ZTL alone is ~€200 a crossing. Castelfalfi and the Amalfi hotel have their own parking, Naples has hotel valet. Budget roughly €60 in tolls from Aug 29 on and a full tank about every 2–3 driving days.</t>
+    <t>You are car-free for the first five days: a private driver in from FCO, taxis and your feet in Rome, the Frecciarossa to Florence. The rental is only collected on Aug 29, on Borgo Ognissanti just outside Florence's ZTL, and returned in Florence again on Sep 1 before the Naples train — three driving days, not fourteen. Everything south of that (Naples, Capri, Amalfi, and the ride back to Rome) is ferry, private driver or train, never a car you're driving yourself. The IDP ships by Aug 3; pack it with the physical licence, not just a photo of it. Never drive into either historic centre — Florence's ZTL alone is ~€200 a crossing. Castelfalfi has its own parking. Budget roughly €40 in tolls for the Florence–Tuscany stretch and a full tank each way.</t>
   </si>
   <si>
     <t>#</t>
@@ -1195,10 +1204,10 @@
     <t>THIS WEEK</t>
   </si>
   <si>
-    <t>Rebook the rental car — Florence pickup, not FCO</t>
-  </si>
-  <si>
-    <t>Reservation #21586310US4 is still FCO Aug 24 → FCO Sep 6. It needs to become Borgo Ognissanti, Florence, Aug 29 → FCO Sep 6: six days shorter, but a different pickup city usually carries a one-way fee, so the €1,087.81 quote will not hold. Re-quote before cancelling. While you are on the phone, move the Sep 6 drop-off off noon — the flight leaves at 10:20am, so around 6:00am.</t>
+    <t>Rebook the rental car — Florence pickup and drop-off, not FCO</t>
+  </si>
+  <si>
+    <t>Reservation #21586310US4 is still FCO Aug 24 → FCO Sep 6. It needs to become Borgo Ognissanti, Florence, Aug 29 → Florence Sep 1: three days rather than fourteen, both ends in the same city. A different pickup/drop-off city usually carries a fee, so the €1,087.81 quote will not hold — re-quote before cancelling.</t>
   </si>
   <si>
     <t>Book the FCO → Hotel Trame private driver</t>
@@ -1237,10 +1246,16 @@
     <t>Three in one morning, in that order. Book the dome climb first; it has the fewest slots.</t>
   </si>
   <si>
-    <t>Vatican early entry (Aug 25), Colosseum arena floor (Aug 26), Pompeii guide (Sep 3)</t>
-  </si>
-  <si>
-    <t>All three need booking — the Vatican and Colosseum slots go first. Pompeii moved to Sep 3 with the reorder; take a morning slot, the site has almost no shade by noon.</t>
+    <t>Vatican early entry (Aug 25), Colosseum arena floor (Aug 26)</t>
+  </si>
+  <si>
+    <t>Both need booking — the Vatican slots go first. Pompeii is dropped from the itinerary, so there's no third guide to book here.</t>
+  </si>
+  <si>
+    <t>Arrange private drivers — Naples → Amalfi (Sep 3) and Amalfi → Naples (Sep 5)</t>
+  </si>
+  <si>
+    <t>No rental car for either leg. Book a local car service for the coast road in both directions — the hotel can usually arrange this directly.</t>
   </si>
   <si>
     <t>Capri ferry — Naples → Capri return, Sep 2</t>
@@ -1258,6 +1273,12 @@
     <t>Festival runs to Sep 5, so both Amalfi nights now fall inside the window. The Aug 29 Mahler date still lands on your Florence→Castelfalfi transfer, so it was never reachable.</t>
   </si>
   <si>
+    <t>Naples → Rome train, Sep 5</t>
+  </si>
+  <si>
+    <t>Frecciarossa runs the route roughly every half hour, about 1h10 — no need to lock this in until closer to the date.</t>
+  </si>
+  <si>
     <t>Headline dinners on their dates</t>
   </si>
   <si>
@@ -1354,7 +1375,7 @@
     <t>~$425 / 60 min</t>
   </si>
   <si>
-    <t>Days 9–11</t>
+    <t>Days 11–13</t>
   </si>
   <si>
     <t>Flytographer Amalfi / Giuseppe Di Martino</t>
@@ -1394,7 +1415,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1447,11 +1468,6 @@
       <b/>
       <color rgb="FF9E4529"/>
       <sz val="8"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF8A6D1F"/>
-      <sz val="9"/>
     </font>
     <font>
       <b/>
@@ -1507,7 +1523,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1533,19 +1549,16 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2072,7 +2085,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F136"/>
+  <dimension ref="A1:F137"/>
   <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -3551,18 +3564,24 @@
         <v>111</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>48</v>
       </c>
       <c r="B86" t="s">
         <v>48</v>
       </c>
-      <c r="C86" t="s">
-        <v>48</v>
-      </c>
-      <c r="D86" s="15" t="s">
+      <c r="C86" s="12" t="s">
         <v>213</v>
+      </c>
+      <c r="D86" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="E86" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="F86" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -3573,13 +3592,13 @@
         <v>48</v>
       </c>
       <c r="C87" s="12" t="s">
-        <v>214</v>
+        <v>183</v>
       </c>
       <c r="D87" s="4" t="s">
         <v>215</v>
       </c>
       <c r="E87" s="13" t="s">
-        <v>165</v>
+        <v>216</v>
       </c>
       <c r="F87" t="s">
         <v>48</v>
@@ -3593,13 +3612,13 @@
         <v>48</v>
       </c>
       <c r="C88" s="12" t="s">
-        <v>216</v>
+        <v>143</v>
       </c>
       <c r="D88" s="4" t="s">
         <v>217</v>
       </c>
       <c r="E88" s="13" t="s">
-        <v>165</v>
+        <v>88</v>
       </c>
       <c r="F88" t="s">
         <v>48</v>
@@ -3613,16 +3632,16 @@
         <v>48</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E89" s="13" t="s">
-        <v>57</v>
+        <v>220</v>
       </c>
       <c r="F89" s="7" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
@@ -3633,16 +3652,16 @@
         <v>48</v>
       </c>
       <c r="C90" s="12" t="s">
-        <v>58</v>
+        <v>221</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E90" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F90" s="7" t="s">
-        <v>77</v>
+        <v>57</v>
+      </c>
+      <c r="F90" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
@@ -3653,16 +3672,16 @@
         <v>48</v>
       </c>
       <c r="C91" s="12" t="s">
-        <v>84</v>
+        <v>223</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="E91" s="13" t="s">
-        <v>221</v>
-      </c>
-      <c r="F91" t="s">
-        <v>48</v>
+        <v>76</v>
+      </c>
+      <c r="F91" s="7" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
@@ -3676,10 +3695,10 @@
         <v>194</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E92" s="13" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="F92" t="s">
         <v>48</v>
@@ -3693,47 +3712,47 @@
         <v>48</v>
       </c>
       <c r="C93" s="12" t="s">
-        <v>132</v>
+        <v>89</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E93" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="F93" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>48</v>
-      </c>
-      <c r="B94" t="s">
-        <v>48</v>
-      </c>
-      <c r="C94" s="12" t="s">
-        <v>224</v>
-      </c>
-      <c r="D94" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="E94" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="F94" s="7" t="s">
+      <c r="F93" s="7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="96" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="10">
+    <row r="95" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="10">
         <v>10</v>
       </c>
-      <c r="B96" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="C96" s="11" t="s">
+      <c r="B95" s="10" t="s">
         <v>227</v>
+      </c>
+      <c r="C95" s="11" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>48</v>
+      </c>
+      <c r="B96" t="s">
+        <v>48</v>
+      </c>
+      <c r="C96" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="E96" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="F96" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
@@ -3744,16 +3763,16 @@
         <v>48</v>
       </c>
       <c r="C97" s="12" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="E97" s="13" t="s">
-        <v>230</v>
-      </c>
-      <c r="F97" t="s">
-        <v>48</v>
+        <v>233</v>
+      </c>
+      <c r="F97" s="7" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -3764,16 +3783,16 @@
         <v>48</v>
       </c>
       <c r="C98" s="12" t="s">
-        <v>231</v>
+        <v>166</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="E98" s="13" t="s">
-        <v>233</v>
-      </c>
-      <c r="F98" s="7" t="s">
-        <v>234</v>
+        <v>236</v>
+      </c>
+      <c r="F98" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -3784,16 +3803,16 @@
         <v>48</v>
       </c>
       <c r="C99" s="12" t="s">
-        <v>166</v>
+        <v>78</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E99" s="13" t="s">
-        <v>236</v>
-      </c>
-      <c r="F99" t="s">
-        <v>48</v>
+        <v>238</v>
+      </c>
+      <c r="F99" s="7" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
@@ -3804,16 +3823,16 @@
         <v>48</v>
       </c>
       <c r="C100" s="12" t="s">
-        <v>78</v>
+        <v>190</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E100" s="13" t="s">
-        <v>238</v>
+        <v>60</v>
       </c>
       <c r="F100" s="7" t="s">
-        <v>71</v>
+        <v>169</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -3824,16 +3843,16 @@
         <v>48</v>
       </c>
       <c r="C101" s="12" t="s">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E101" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="F101" s="7" t="s">
-        <v>169</v>
+        <v>233</v>
+      </c>
+      <c r="F101" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -3844,50 +3863,50 @@
         <v>48</v>
       </c>
       <c r="C102" s="12" t="s">
-        <v>240</v>
+        <v>89</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E102" s="13" t="s">
-        <v>233</v>
-      </c>
-      <c r="F102" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>48</v>
-      </c>
-      <c r="B103" t="s">
-        <v>48</v>
-      </c>
-      <c r="C103" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="D103" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="E103" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="F103" s="7" t="s">
+      <c r="F102" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="105" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="10">
+    <row r="104" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="10">
         <v>11</v>
       </c>
-      <c r="B105" s="10" t="s">
+      <c r="B104" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="C105" s="11" t="s">
+      <c r="C104" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="F105" s="14" t="s">
+      <c r="F104" s="14" t="s">
         <v>111</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>48</v>
+      </c>
+      <c r="B105" t="s">
+        <v>48</v>
+      </c>
+      <c r="C105" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="E105" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="F105" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
@@ -3898,13 +3917,13 @@
         <v>48</v>
       </c>
       <c r="C106" s="12" t="s">
-        <v>228</v>
+        <v>112</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E106" s="13" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="F106" t="s">
         <v>48</v>
@@ -3918,13 +3937,13 @@
         <v>48</v>
       </c>
       <c r="C107" s="12" t="s">
-        <v>246</v>
+        <v>143</v>
       </c>
       <c r="D107" s="4" t="s">
         <v>247</v>
       </c>
       <c r="E107" s="13" t="s">
-        <v>248</v>
+        <v>63</v>
       </c>
       <c r="F107" t="s">
         <v>48</v>
@@ -3938,16 +3957,16 @@
         <v>48</v>
       </c>
       <c r="C108" s="12" t="s">
-        <v>183</v>
+        <v>145</v>
       </c>
       <c r="D108" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="E108" s="13" t="s">
         <v>249</v>
       </c>
-      <c r="E108" s="13" t="s">
-        <v>250</v>
-      </c>
-      <c r="F108" s="7" t="s">
-        <v>77</v>
+      <c r="F108" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
@@ -3958,16 +3977,16 @@
         <v>48</v>
       </c>
       <c r="C109" s="12" t="s">
-        <v>78</v>
+        <v>203</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E109" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="F109" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="F109" s="7" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
@@ -3981,13 +4000,13 @@
         <v>58</v>
       </c>
       <c r="D110" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="E110" s="13" t="s">
         <v>252</v>
       </c>
-      <c r="E110" s="13" t="s">
-        <v>253</v>
-      </c>
-      <c r="F110" s="7" t="s">
-        <v>123</v>
+      <c r="F110" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -3998,13 +4017,13 @@
         <v>48</v>
       </c>
       <c r="C111" s="12" t="s">
-        <v>84</v>
+        <v>253</v>
       </c>
       <c r="D111" s="4" t="s">
         <v>254</v>
       </c>
       <c r="E111" s="13" t="s">
-        <v>255</v>
+        <v>63</v>
       </c>
       <c r="F111" t="s">
         <v>48</v>
@@ -4018,47 +4037,47 @@
         <v>48</v>
       </c>
       <c r="C112" s="12" t="s">
-        <v>256</v>
+        <v>107</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E112" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="F112" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>48</v>
-      </c>
-      <c r="B113" t="s">
-        <v>48</v>
-      </c>
-      <c r="C113" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="D113" s="4" t="s">
+      <c r="F112" s="7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="114" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="10">
+        <v>12</v>
+      </c>
+      <c r="B114" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="C114" s="11" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>48</v>
+      </c>
+      <c r="B115" t="s">
+        <v>48</v>
+      </c>
+      <c r="C115" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="D115" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="E113" s="13" t="s">
+      <c r="E115" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="F113" s="7" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="115" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="10">
-        <v>12</v>
-      </c>
-      <c r="B115" s="10" t="s">
-        <v>259</v>
-      </c>
-      <c r="C115" s="11" t="s">
-        <v>260</v>
+      <c r="F115" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
@@ -4069,16 +4088,16 @@
         <v>48</v>
       </c>
       <c r="C116" s="12" t="s">
-        <v>161</v>
+        <v>186</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E116" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="F116" t="s">
-        <v>48</v>
+        <v>260</v>
+      </c>
+      <c r="F116" s="7" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
@@ -4089,16 +4108,16 @@
         <v>48</v>
       </c>
       <c r="C117" s="12" t="s">
-        <v>186</v>
+        <v>58</v>
       </c>
       <c r="D117" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="E117" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="E117" s="13" t="s">
-        <v>263</v>
-      </c>
-      <c r="F117" s="7" t="s">
-        <v>71</v>
+      <c r="F117" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
@@ -4109,16 +4128,16 @@
         <v>48</v>
       </c>
       <c r="C118" s="12" t="s">
-        <v>58</v>
+        <v>263</v>
       </c>
       <c r="D118" s="4" t="s">
         <v>264</v>
       </c>
       <c r="E118" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="F118" t="s">
-        <v>48</v>
+        <v>265</v>
+      </c>
+      <c r="F118" s="7" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
@@ -4129,13 +4148,13 @@
         <v>48</v>
       </c>
       <c r="C119" s="12" t="s">
-        <v>265</v>
+        <v>194</v>
       </c>
       <c r="D119" s="4" t="s">
         <v>266</v>
       </c>
       <c r="E119" s="13" t="s">
-        <v>267</v>
+        <v>88</v>
       </c>
       <c r="F119" s="7" t="s">
         <v>77</v>
@@ -4149,16 +4168,16 @@
         <v>48</v>
       </c>
       <c r="C120" s="12" t="s">
-        <v>194</v>
+        <v>64</v>
       </c>
       <c r="D120" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="E120" s="13" t="s">
         <v>268</v>
       </c>
-      <c r="E120" s="13" t="s">
-        <v>88</v>
-      </c>
       <c r="F120" s="7" t="s">
-        <v>77</v>
+        <v>269</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
@@ -4169,50 +4188,50 @@
         <v>48</v>
       </c>
       <c r="C121" s="12" t="s">
-        <v>64</v>
+        <v>270</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E121" s="13" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F121" s="7" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>48</v>
-      </c>
-      <c r="B122" t="s">
-        <v>48</v>
-      </c>
-      <c r="C122" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="D122" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="123" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A123" s="10">
+        <v>13</v>
+      </c>
+      <c r="B123" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="E122" s="13" t="s">
+      <c r="C123" s="11" t="s">
         <v>274</v>
       </c>
-      <c r="F122" s="7" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="124" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="10">
-        <v>13</v>
-      </c>
-      <c r="B124" s="10" t="s">
+      <c r="F123" s="14" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>48</v>
+      </c>
+      <c r="B124" t="s">
+        <v>48</v>
+      </c>
+      <c r="C124" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="D124" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="C124" s="11" t="s">
-        <v>276</v>
-      </c>
-      <c r="F124" s="14" t="s">
-        <v>111</v>
+      <c r="E124" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="F124" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
@@ -4223,13 +4242,13 @@
         <v>48</v>
       </c>
       <c r="C125" s="12" t="s">
-        <v>228</v>
+        <v>112</v>
       </c>
       <c r="D125" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="E125" s="13" t="s">
         <v>277</v>
-      </c>
-      <c r="E125" s="13" t="s">
-        <v>63</v>
       </c>
       <c r="F125" t="s">
         <v>48</v>
@@ -4243,13 +4262,13 @@
         <v>48</v>
       </c>
       <c r="C126" s="12" t="s">
-        <v>112</v>
+        <v>143</v>
       </c>
       <c r="D126" s="4" t="s">
         <v>278</v>
       </c>
       <c r="E126" s="13" t="s">
-        <v>165</v>
+        <v>57</v>
       </c>
       <c r="F126" t="s">
         <v>48</v>
@@ -4263,16 +4282,16 @@
         <v>48</v>
       </c>
       <c r="C127" s="12" t="s">
-        <v>203</v>
+        <v>49</v>
       </c>
       <c r="D127" s="4" t="s">
         <v>279</v>
       </c>
       <c r="E127" s="13" t="s">
-        <v>57</v>
+        <v>220</v>
       </c>
       <c r="F127" s="7" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
@@ -4283,13 +4302,13 @@
         <v>48</v>
       </c>
       <c r="C128" s="12" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="D128" s="4" t="s">
         <v>280</v>
       </c>
       <c r="E128" s="13" t="s">
-        <v>230</v>
+        <v>76</v>
       </c>
       <c r="F128" t="s">
         <v>48</v>
@@ -4303,16 +4322,16 @@
         <v>48</v>
       </c>
       <c r="C129" s="12" t="s">
-        <v>61</v>
+        <v>203</v>
       </c>
       <c r="D129" s="4" t="s">
         <v>281</v>
       </c>
       <c r="E129" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="F129" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="F129" s="7" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
@@ -4323,61 +4342,67 @@
         <v>48</v>
       </c>
       <c r="C130" s="12" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="D130" s="4" t="s">
         <v>282</v>
       </c>
       <c r="E130" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="F130" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>48</v>
+      </c>
+      <c r="B131" t="s">
+        <v>48</v>
+      </c>
+      <c r="C131" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="D131" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="E131" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="F131" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>48</v>
+      </c>
+      <c r="B132" t="s">
+        <v>48</v>
+      </c>
+      <c r="C132" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D132" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="E132" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="F130" s="7" t="s">
+      <c r="F132" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="132" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="10">
+    <row r="134" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A134" s="10">
         <v>14</v>
       </c>
-      <c r="B132" s="10" t="s">
-        <v>283</v>
-      </c>
-      <c r="C132" s="11" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A133" t="s">
-        <v>48</v>
-      </c>
-      <c r="B133" t="s">
-        <v>48</v>
-      </c>
-      <c r="C133" t="s">
-        <v>48</v>
-      </c>
-      <c r="D133" s="15" t="s">
+      <c r="B134" s="10" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
-        <v>48</v>
-      </c>
-      <c r="B134" t="s">
-        <v>48</v>
-      </c>
-      <c r="C134" s="12" t="s">
+      <c r="C134" s="11" t="s">
         <v>286</v>
-      </c>
-      <c r="D134" s="4" t="s">
-        <v>287</v>
-      </c>
-      <c r="E134" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="F134" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
@@ -4388,13 +4413,13 @@
         <v>48</v>
       </c>
       <c r="C135" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="D135" s="4" t="s">
         <v>288</v>
       </c>
-      <c r="D135" s="4" t="s">
-        <v>289</v>
-      </c>
       <c r="E135" s="13" t="s">
-        <v>290</v>
+        <v>83</v>
       </c>
       <c r="F135" t="s">
         <v>48</v>
@@ -4408,15 +4433,35 @@
         <v>48</v>
       </c>
       <c r="C136" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="D136" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="E136" s="13" t="s">
         <v>291</v>
       </c>
-      <c r="D136" s="4" t="s">
+      <c r="F136" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>48</v>
+      </c>
+      <c r="B137" t="s">
+        <v>48</v>
+      </c>
+      <c r="C137" s="12" t="s">
         <v>292</v>
       </c>
-      <c r="E136" s="13" t="s">
+      <c r="D137" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="F136" t="s">
+      <c r="E137" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="F137" t="s">
         <v>48</v>
       </c>
     </row>
@@ -4447,22 +4492,22 @@
     <hyperlink ref="F54" r:id="rId23"/>
     <hyperlink ref="F58" r:id="rId24"/>
     <hyperlink ref="F89" r:id="rId25"/>
-    <hyperlink ref="F90" r:id="rId26"/>
-    <hyperlink ref="F94" r:id="rId27"/>
-    <hyperlink ref="F98" r:id="rId28"/>
-    <hyperlink ref="F100" r:id="rId29"/>
-    <hyperlink ref="F101" r:id="rId30"/>
-    <hyperlink ref="F103" r:id="rId31"/>
-    <hyperlink ref="F108" r:id="rId32"/>
-    <hyperlink ref="F110" r:id="rId33"/>
-    <hyperlink ref="F113" r:id="rId34"/>
-    <hyperlink ref="F117" r:id="rId35"/>
+    <hyperlink ref="F91" r:id="rId26"/>
+    <hyperlink ref="F93" r:id="rId27"/>
+    <hyperlink ref="F97" r:id="rId28"/>
+    <hyperlink ref="F99" r:id="rId29"/>
+    <hyperlink ref="F100" r:id="rId30"/>
+    <hyperlink ref="F102" r:id="rId31"/>
+    <hyperlink ref="F109" r:id="rId32"/>
+    <hyperlink ref="F112" r:id="rId33"/>
+    <hyperlink ref="F116" r:id="rId34"/>
+    <hyperlink ref="F118" r:id="rId35"/>
     <hyperlink ref="F119" r:id="rId36"/>
     <hyperlink ref="F120" r:id="rId37"/>
     <hyperlink ref="F121" r:id="rId38"/>
-    <hyperlink ref="F122" r:id="rId39"/>
-    <hyperlink ref="F127" r:id="rId40"/>
-    <hyperlink ref="F130" r:id="rId41"/>
+    <hyperlink ref="F127" r:id="rId39"/>
+    <hyperlink ref="F129" r:id="rId40"/>
+    <hyperlink ref="F132" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -4485,42 +4530,42 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D2" t="s">
         <v>46</v>
@@ -4531,10 +4576,10 @@
       <c r="F2">
         <v>3</v>
       </c>
-      <c r="G2" s="16">
+      <c r="G2" s="15">
         <v>523.86</v>
       </c>
-      <c r="H2" s="16">
+      <c r="H2" s="15">
         <v>1571.58</v>
       </c>
       <c r="I2" s="7" t="s">
@@ -4543,13 +4588,13 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B3" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D3" t="s">
         <v>109</v>
@@ -4560,10 +4605,10 @@
       <c r="F3">
         <v>2</v>
       </c>
-      <c r="G3" s="16">
+      <c r="G3" s="15">
         <v>735</v>
       </c>
-      <c r="H3" s="16">
+      <c r="H3" s="15">
         <v>1470</v>
       </c>
       <c r="I3" s="7" t="s">
@@ -4572,13 +4617,13 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B4" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C4" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D4" t="s">
         <v>159</v>
@@ -4589,10 +4634,10 @@
       <c r="F4">
         <v>3</v>
       </c>
-      <c r="G4" s="16">
+      <c r="G4" s="15">
         <v>1254.99</v>
       </c>
-      <c r="H4" s="16">
+      <c r="H4" s="15">
         <v>3764.98</v>
       </c>
       <c r="I4" s="7" t="s">
@@ -4601,13 +4646,13 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B5" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C5" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D5" t="s">
         <v>211</v>
@@ -4618,11 +4663,11 @@
       <c r="F5">
         <v>2</v>
       </c>
-      <c r="G5" s="16">
-        <v>549.14</v>
-      </c>
-      <c r="H5" s="16">
-        <v>1098.27</v>
+      <c r="G5" s="15">
+        <v>535.5</v>
+      </c>
+      <c r="H5" s="15">
+        <v>1071</v>
       </c>
       <c r="I5" s="7" t="s">
         <v>123</v>
@@ -4630,27 +4675,27 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D6" t="s">
         <v>243</v>
       </c>
       <c r="E6" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="15">
         <v>1500</v>
       </c>
-      <c r="H6" s="16">
+      <c r="H6" s="15">
         <v>3000</v>
       </c>
       <c r="I6" s="7" t="s">
@@ -4659,57 +4704,57 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B7" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C7" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D7" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="E7" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="15">
         <v>1000</v>
       </c>
-      <c r="H7" s="16">
+      <c r="H7" s="15">
         <v>1000</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>321</v>
-      </c>
-      <c r="F8" s="17">
+    <row r="8" spans="1:8" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>322</v>
+      </c>
+      <c r="F8" s="16">
         <v>13</v>
       </c>
-      <c r="G8" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" s="18">
-        <v>11904.83</v>
+      <c r="G8" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" s="17">
+        <v>11877.56</v>
       </c>
     </row>
   </sheetData>
@@ -4738,79 +4783,79 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>325</v>
-      </c>
-      <c r="B2" s="16">
-        <v>11904.83</v>
+        <v>326</v>
+      </c>
+      <c r="B2" s="15">
+        <v>11877.56</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="16">
+      <c r="B3" s="15">
         <v>1775</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>328</v>
-      </c>
-      <c r="B4" s="16">
-        <v>2100</v>
+        <v>329</v>
+      </c>
+      <c r="B4" s="15">
+        <v>1900</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>330</v>
-      </c>
-      <c r="B5" s="16">
+        <v>331</v>
+      </c>
+      <c r="B5" s="15">
         <v>2400</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>332</v>
-      </c>
-      <c r="B6" s="16">
+        <v>333</v>
+      </c>
+      <c r="B6" s="15">
         <v>400</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="17" t="s">
-        <v>321</v>
-      </c>
-      <c r="B7" s="18">
-        <v>18579.83</v>
-      </c>
-      <c r="C7" s="17" t="s">
         <v>334</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="16" t="s">
+        <v>322</v>
+      </c>
+      <c r="B7" s="17">
+        <v>18352.559999999998</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -4821,7 +4866,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -4835,26 +4880,26 @@
         <v>41</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B2" t="s">
-        <v>339</v>
-      </c>
-      <c r="C2" s="19" t="s">
+        <v>262</v>
+      </c>
+      <c r="C2" s="18" t="s">
         <v>340</v>
       </c>
       <c r="D2" t="s">
@@ -4871,7 +4916,7 @@
       <c r="B3" t="s">
         <v>344</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>345</v>
       </c>
       <c r="D3" t="s">
@@ -4888,7 +4933,7 @@
       <c r="B4" t="s">
         <v>348</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>349</v>
       </c>
       <c r="D4" t="s">
@@ -4905,7 +4950,7 @@
       <c r="B5" t="s">
         <v>165</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>351</v>
       </c>
       <c r="D5" t="s">
@@ -4922,7 +4967,7 @@
       <c r="B6" t="s">
         <v>354</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>355</v>
       </c>
       <c r="D6" t="s">
@@ -4939,7 +4984,7 @@
       <c r="B7" t="s">
         <v>358</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>359</v>
       </c>
       <c r="D7" t="s">
@@ -4954,13 +4999,13 @@
         <v>361</v>
       </c>
       <c r="B8" t="s">
-        <v>165</v>
-      </c>
-      <c r="C8" s="19" t="s">
         <v>362</v>
       </c>
+      <c r="C8" s="18" t="s">
+        <v>363</v>
+      </c>
       <c r="D8" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>342</v>
@@ -4968,16 +5013,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B9" t="s">
-        <v>365</v>
-      </c>
-      <c r="C9" s="19" t="s">
         <v>366</v>
       </c>
+      <c r="C9" s="18" t="s">
+        <v>367</v>
+      </c>
       <c r="D9" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>342</v>
@@ -4985,16 +5030,16 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B10" t="s">
-        <v>165</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>369</v>
+        <v>262</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>370</v>
       </c>
       <c r="D10" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>342</v>
@@ -5002,16 +5047,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B11" t="s">
-        <v>165</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>372</v>
+        <v>262</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>373</v>
       </c>
       <c r="D11" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>342</v>
@@ -5019,16 +5064,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B12" t="s">
-        <v>165</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>374</v>
+        <v>262</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>376</v>
       </c>
       <c r="D12" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>342</v>
@@ -5036,12 +5081,12 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B13" t="s">
-        <v>377</v>
-      </c>
-      <c r="C13" s="19" t="s">
+        <v>220</v>
+      </c>
+      <c r="C13" s="18" t="s">
         <v>378</v>
       </c>
       <c r="D13" t="s">
@@ -5051,314 +5096,32 @@
         <v>342</v>
       </c>
     </row>
-    <row r="15" ht="44" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" t="s">
-        <v>48</v>
-      </c>
-      <c r="C15" s="4" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>380</v>
       </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1"/>
-    <hyperlink ref="E3" r:id="rId2"/>
-    <hyperlink ref="E4" r:id="rId3"/>
-    <hyperlink ref="E5" r:id="rId4"/>
-    <hyperlink ref="E6" r:id="rId5"/>
-    <hyperlink ref="E7" r:id="rId6"/>
-    <hyperlink ref="E8" r:id="rId7"/>
-    <hyperlink ref="E9" r:id="rId8"/>
-    <hyperlink ref="E10" r:id="rId9"/>
-    <hyperlink ref="E11" r:id="rId10"/>
-    <hyperlink ref="E12" r:id="rId11"/>
-    <hyperlink ref="E13" r:id="rId12"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E18"/>
-  <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="3" width="68" customWidth="1"/>
-    <col min="4" max="5" width="14" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="B14" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" s="18" t="s">
         <v>381</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="D14" t="s">
         <v>382</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="E14" s="7" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="16" ht="44" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>383</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>384</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>385</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>386</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>387</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>390</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>391</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>392</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>393</v>
-      </c>
-      <c r="D4" s="20" t="s">
-        <v>387</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>394</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>395</v>
-      </c>
-      <c r="D5" s="20" t="s">
-        <v>387</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>396</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>397</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>387</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>398</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>399</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>391</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>400</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>401</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>391</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>402</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>391</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>404</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>405</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>391</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>406</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>407</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>391</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>408</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>409</v>
-      </c>
-      <c r="D12" s="22" t="s">
-        <v>410</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>411</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>412</v>
-      </c>
-      <c r="D13" s="22" t="s">
-        <v>410</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>413</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>414</v>
-      </c>
-      <c r="D14" s="22" t="s">
-        <v>410</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>48</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>48</v>
-      </c>
-      <c r="B17" s="24" t="s">
-        <v>416</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="24" t="s">
-        <v>418</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>419</v>
       </c>
     </row>
   </sheetData>
@@ -5376,6 +5139,342 @@
     <hyperlink ref="E12" r:id="rId11"/>
     <hyperlink ref="E13" r:id="rId12"/>
     <hyperlink ref="E14" r:id="rId13"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="52" customWidth="1"/>
+    <col min="3" max="3" width="68" customWidth="1"/>
+    <col min="4" max="5" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>384</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>385</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>386</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>387</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>390</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>394</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>390</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>397</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>390</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>390</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>394</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>394</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>394</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>394</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>410</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>394</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>394</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>415</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>415</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>415</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>415</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>423</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="23" t="s">
+        <v>425</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1"/>
+    <hyperlink ref="E3" r:id="rId2"/>
+    <hyperlink ref="E4" r:id="rId3"/>
+    <hyperlink ref="E5" r:id="rId4"/>
+    <hyperlink ref="E6" r:id="rId5"/>
+    <hyperlink ref="E7" r:id="rId6"/>
+    <hyperlink ref="E8" r:id="rId7"/>
+    <hyperlink ref="E9" r:id="rId8"/>
+    <hyperlink ref="E10" r:id="rId9"/>
+    <hyperlink ref="E11" r:id="rId10"/>
+    <hyperlink ref="E12" r:id="rId11"/>
+    <hyperlink ref="E13" r:id="rId12"/>
+    <hyperlink ref="E14" r:id="rId13"/>
+    <hyperlink ref="E15" r:id="rId14"/>
+    <hyperlink ref="E16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -5398,158 +5497,158 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B2" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="C2" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="E2" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="F2" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B3" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="C3" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="E3" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="F3" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="B4" t="s">
+        <v>447</v>
+      </c>
+      <c r="C4" t="s">
+        <v>448</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="E4" t="s">
+        <v>450</v>
+      </c>
+      <c r="F4" t="s">
+        <v>451</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>440</v>
       </c>
-      <c r="C4" t="s">
+      <c r="H4" s="7" t="s">
         <v>441</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>442</v>
-      </c>
-      <c r="E4" t="s">
-        <v>443</v>
-      </c>
-      <c r="F4" t="s">
-        <v>444</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>433</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>434</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B5" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="C5" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="E5" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="F5" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="B6" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="C6" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
       <c r="E6" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="F6" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5563,7 +5662,7 @@
         <v>48</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Move Villa Borghese from evening museum ticket to daytime garden photos
Day 3 was the only Rome day with room: the arrival day is protected
jet-lag recovery and Day 2 (Vatican) is already full through a late
dinner. Swaps the near-dark 7pm optional Galleria Borghese slot for
actual daylight at the gardens and Pincio terrace, no ticket needed;
Trastevere shifts later to take the evening instead.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/italy-2026/dist/Italy 2026 (revised).xlsx
+++ b/italy-2026/dist/Italy 2026 (revised).xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1003" uniqueCount="465">
   <si>
     <t>ITALY 2026 PLAN</t>
   </si>
@@ -322,237 +322,249 @@
     <t>Walk, 5 min via Campo de' Fiori</t>
   </si>
   <si>
-    <t>Siesta</t>
+    <t>Siesta — Shorter than the other days — the light at Borghese is worth trading a bit of rest for</t>
+  </si>
+  <si>
+    <t>4:00pm</t>
+  </si>
+  <si>
+    <t>Villa Borghese Gardens, in the daylight — Rome's largest park — shaded avenues, the Fontana dei Cavalli Marini, and the Pincio terrace over Piazza del Popolo with St. Peter's dome on the skyline. Soft light under the trees most of the afternoon — good ground for pictures. The Galleria itself needs a timed ticket booked weeks out; skip it unless you already have one.</t>
+  </si>
+  <si>
+    <t>Info -&gt;</t>
+  </si>
+  <si>
+    <t>5:30pm</t>
+  </si>
+  <si>
+    <t>Down to Piazza del Popolo — The twin churches and the obelisk, down the Pincio steps</t>
+  </si>
+  <si>
+    <t>Walk down, ~10 min</t>
+  </si>
+  <si>
+    <t>6:15pm</t>
   </si>
   <si>
     <t>Trastevere on foot — Cross the Tiber and wander to Piazza Santa Maria in Trastevere</t>
   </si>
   <si>
+    <t>9:00pm</t>
+  </si>
+  <si>
+    <t>Dinner — Da Enzo al 29 — Trastevere, twelve tables, no reservations after 9pm</t>
+  </si>
+  <si>
     <t>Walk, ~12 min</t>
   </si>
   <si>
+    <t>Thu, Aug 27</t>
+  </si>
+  <si>
+    <t>ROME → FLORENCE — Casa G. Firenze</t>
+  </si>
+  <si>
+    <t>TRAVEL DAY</t>
+  </si>
+  <si>
+    <t>9:30am</t>
+  </si>
+  <si>
+    <t>Check out; taxi to Roma Termini — About fifteen minutes from Campo de' Fiori. Aim to be at the platform twenty minutes before departure.</t>
+  </si>
+  <si>
+    <t>10:35am</t>
+  </si>
+  <si>
+    <t>Frecciarossa — Roma Termini → Firenze S.M.N. — Book Trenitalia or Italo well ahead; advance fares are a fraction of the walk-up price and both run the route hourly.</t>
+  </si>
+  <si>
+    <t>High-speed rail, ~1h30</t>
+  </si>
+  <si>
+    <t>Trenitalia -&gt;</t>
+  </si>
+  <si>
+    <t>12:10pm</t>
+  </si>
+  <si>
+    <t>Arrive Firenze Santa Maria Novella — The station is a nine-minute walk from Via dei Rondinelli — no transfer needed</t>
+  </si>
+  <si>
+    <t>Walk, ~9 min</t>
+  </si>
+  <si>
+    <t>12:45pm</t>
+  </si>
+  <si>
+    <t>Drop bags at Casa G. Firenze — Via dei Rondinelli, between the Duomo and Santa Maria Novella. Rooms are ready from 3:00pm; they will hold luggage until then.</t>
+  </si>
+  <si>
+    <t>Trip.com -&gt;</t>
+  </si>
+  <si>
+    <t>1:15pm</t>
+  </si>
+  <si>
+    <t>Lunch at the Mercato Centrale — Five minutes north — the upstairs food hall, no booking, no ceremony</t>
+  </si>
+  <si>
+    <t>Walk, ~5 min</t>
+  </si>
+  <si>
+    <t>2:45pm</t>
+  </si>
+  <si>
+    <t>First orientation walk — The Duomo and Baptistery from the outside, then Piazza della Repubblica and down to the Arno. The ticketed interiors are all tomorrow — today is just getting your bearings.</t>
+  </si>
+  <si>
+    <t>Unpack and reset — The train bought you an afternoon the drive would have eaten</t>
+  </si>
+  <si>
+    <t>6:45pm</t>
+  </si>
+  <si>
+    <t>Aperitivo on the secret patio — Casa G.'s courtyard bar</t>
+  </si>
+  <si>
+    <t>8:00pm</t>
+  </si>
+  <si>
+    <t>OPERA — La Traviata at St. Mark's Anglican — Via Maggio, across Ponte Santa Trinita — booked for arrival evening, comfortably clear now the train lands you at midday.</t>
+  </si>
+  <si>
+    <t>Walk, ~10 min</t>
+  </si>
+  <si>
+    <t>9:45pm</t>
+  </si>
+  <si>
+    <t>Dinner — Trattoria Sostanza — Cash only. The butter chicken and the tortino. Alternative: Buca dell'Orafo.</t>
+  </si>
+  <si>
+    <t>Fri, Aug 28</t>
+  </si>
+  <si>
+    <t>FLORENCE — the full day</t>
+  </si>
+  <si>
+    <t>8:15am</t>
+  </si>
+  <si>
+    <t>Accademia — David at first entry — Forty-five minutes is genuinely enough. Go straight down the hall.</t>
+  </si>
+  <si>
+    <t>Duomo — climb Brunelleschi's dome — 463 steps, timed slot, and much better before the day heats up</t>
+  </si>
+  <si>
+    <t>Walk, ~6 min</t>
+  </si>
+  <si>
+    <t>11:00am</t>
+  </si>
+  <si>
+    <t>Coffee on Piazza della Signoria — The Loggia dei Lanzi is an open-air sculpture hall and it is free</t>
+  </si>
+  <si>
+    <t>11:30am</t>
+  </si>
+  <si>
+    <t>Uffizi, guided — Botticelli, Leonardo, the Caravaggio room. Roughly two hours with a guide.</t>
+  </si>
+  <si>
+    <t>Walk, ~3 min</t>
+  </si>
+  <si>
+    <t>1:45pm</t>
+  </si>
+  <si>
+    <t>Lunch in the Oltrarno — Il Santo Bevitore — Or Gucci Osteria if you want the splurge. Trattoria Mario is the third option if you'd rather eat near San Lorenzo.</t>
+  </si>
+  <si>
+    <t>Cross Ponte Santa Trinita, ~8 min</t>
+  </si>
+  <si>
+    <t>3:15pm</t>
+  </si>
+  <si>
+    <t>Pitti Palace and the Boboli Gardens — The gardens are the reason to go; climb to the top for the view back over the city</t>
+  </si>
+  <si>
+    <t>Oltrarno artisan workshops — Via Maggio and Santo Spirito — gilders, leatherworkers, restorers still working street level</t>
+  </si>
+  <si>
+    <t>7:15pm</t>
+  </si>
+  <si>
+    <t>Ponte Vecchio, then up to Piazzale Michelangelo — Sunset is around 8:00pm. Taxi up, walk down.</t>
+  </si>
+  <si>
+    <t>Taxi up, ~10 min</t>
+  </si>
+  <si>
+    <t>Dinner — Borgo San Jacopo — Michelin-starred, on the river, with a handful of window tables. Ask for one.</t>
+  </si>
+  <si>
+    <t>Walk down, ~15 min</t>
+  </si>
+  <si>
+    <t>Sat, Aug 29</t>
+  </si>
+  <si>
+    <t>FLORENCE → TUSCANY — Il Castelfalfi</t>
+  </si>
+  <si>
+    <t>9:00am</t>
+  </si>
+  <si>
+    <t>Check out; collect the rental car — The agencies cluster on Borgo Ognissanti, ~10 min on foot and just outside the ZTL — so you never drive into the centro storico. Have the IDP and licence ready.</t>
+  </si>
+  <si>
+    <t>9:45am</t>
+  </si>
+  <si>
+    <t>Southwest out of the city — Florence → Certaldo is about 45 minutes</t>
+  </si>
+  <si>
+    <t>Self-drive</t>
+  </si>
+  <si>
+    <t>10:30am</t>
+  </si>
+  <si>
+    <t>Certaldo Alto, by funicular — Boccaccio's birthplace — a walled brick town, the funicular climbs from Piazza Boccaccio in under two minutes</t>
+  </si>
+  <si>
+    <t>Arrive Certaldo</t>
+  </si>
+  <si>
+    <t>11:15am</t>
+  </si>
+  <si>
+    <t>Casa Boccaccio — The Decameron's author was born here; the house is now a small, quiet museum</t>
+  </si>
+  <si>
+    <t>Lunch on Via Boccaccio — A terrace table in the upper town before the drive on</t>
+  </si>
+  <si>
+    <t>On to Castelfalfi — About twenty-five minutes further into the Val d'Elsa</t>
+  </si>
+  <si>
+    <t>Driver</t>
+  </si>
+  <si>
+    <t>Check in — Il Castelfalfi — A restored 14th-century hamlet on a 2,700-acre estate, its own castle at the centre</t>
+  </si>
+  <si>
+    <t>Book -&gt;</t>
+  </si>
+  <si>
+    <t>The hamlet on foot — The piazza, the castle walls, the little church — all restored, none of it roped off</t>
+  </si>
+  <si>
     <t>7:00pm</t>
   </si>
   <si>
-    <t>[optional] Optional — Galleria Borghese — Timed entry, two-hour slots, books out early. Skip it guilt-free if the day already feels long.</t>
-  </si>
-  <si>
-    <t>Taxi, ~20 min</t>
-  </si>
-  <si>
-    <t>9:00pm</t>
-  </si>
-  <si>
-    <t>Dinner — Da Enzo al 29 — Trastevere, twelve tables, no reservations after 9pm</t>
-  </si>
-  <si>
-    <t>Thu, Aug 27</t>
-  </si>
-  <si>
-    <t>ROME → FLORENCE — Casa G. Firenze</t>
-  </si>
-  <si>
-    <t>TRAVEL DAY</t>
-  </si>
-  <si>
-    <t>9:30am</t>
-  </si>
-  <si>
-    <t>Check out; taxi to Roma Termini — About fifteen minutes from Campo de' Fiori. Aim to be at the platform twenty minutes before departure.</t>
-  </si>
-  <si>
-    <t>10:35am</t>
-  </si>
-  <si>
-    <t>Frecciarossa — Roma Termini → Firenze S.M.N. — Book Trenitalia or Italo well ahead; advance fares are a fraction of the walk-up price and both run the route hourly.</t>
-  </si>
-  <si>
-    <t>High-speed rail, ~1h30</t>
-  </si>
-  <si>
-    <t>Trenitalia -&gt;</t>
-  </si>
-  <si>
-    <t>12:10pm</t>
-  </si>
-  <si>
-    <t>Arrive Firenze Santa Maria Novella — The station is a nine-minute walk from Via dei Rondinelli — no transfer needed</t>
-  </si>
-  <si>
-    <t>Walk, ~9 min</t>
-  </si>
-  <si>
-    <t>12:45pm</t>
-  </si>
-  <si>
-    <t>Drop bags at Casa G. Firenze — Via dei Rondinelli, between the Duomo and Santa Maria Novella. Rooms are ready from 3:00pm; they will hold luggage until then.</t>
-  </si>
-  <si>
-    <t>Trip.com -&gt;</t>
-  </si>
-  <si>
-    <t>1:15pm</t>
-  </si>
-  <si>
-    <t>Lunch at the Mercato Centrale — Five minutes north — the upstairs food hall, no booking, no ceremony</t>
-  </si>
-  <si>
-    <t>Walk, ~5 min</t>
-  </si>
-  <si>
-    <t>2:45pm</t>
-  </si>
-  <si>
-    <t>First orientation walk — The Duomo and Baptistery from the outside, then Piazza della Repubblica and down to the Arno. The ticketed interiors are all tomorrow — today is just getting your bearings.</t>
-  </si>
-  <si>
-    <t>Unpack and reset — The train bought you an afternoon the drive would have eaten</t>
-  </si>
-  <si>
-    <t>6:45pm</t>
-  </si>
-  <si>
-    <t>Aperitivo on the secret patio — Casa G.'s courtyard bar</t>
-  </si>
-  <si>
-    <t>8:00pm</t>
-  </si>
-  <si>
-    <t>OPERA — La Traviata at St. Mark's Anglican — Via Maggio, across Ponte Santa Trinita — booked for arrival evening, comfortably clear now the train lands you at midday.</t>
-  </si>
-  <si>
-    <t>Walk, ~10 min</t>
-  </si>
-  <si>
-    <t>9:45pm</t>
-  </si>
-  <si>
-    <t>Dinner — Trattoria Sostanza — Cash only. The butter chicken and the tortino. Alternative: Buca dell'Orafo.</t>
-  </si>
-  <si>
-    <t>Fri, Aug 28</t>
-  </si>
-  <si>
-    <t>FLORENCE — the full day</t>
-  </si>
-  <si>
-    <t>8:15am</t>
-  </si>
-  <si>
-    <t>Accademia — David at first entry — Forty-five minutes is genuinely enough. Go straight down the hall.</t>
-  </si>
-  <si>
-    <t>Duomo — climb Brunelleschi's dome — 463 steps, timed slot, and much better before the day heats up</t>
-  </si>
-  <si>
-    <t>Walk, ~6 min</t>
-  </si>
-  <si>
-    <t>11:00am</t>
-  </si>
-  <si>
-    <t>Coffee on Piazza della Signoria — The Loggia dei Lanzi is an open-air sculpture hall and it is free</t>
-  </si>
-  <si>
-    <t>11:30am</t>
-  </si>
-  <si>
-    <t>Uffizi, guided — Botticelli, Leonardo, the Caravaggio room. Roughly two hours with a guide.</t>
-  </si>
-  <si>
-    <t>Walk, ~3 min</t>
-  </si>
-  <si>
-    <t>1:45pm</t>
-  </si>
-  <si>
-    <t>Lunch in the Oltrarno — Il Santo Bevitore — Or Gucci Osteria if you want the splurge. Trattoria Mario is the third option if you'd rather eat near San Lorenzo.</t>
-  </si>
-  <si>
-    <t>Cross Ponte Santa Trinita, ~8 min</t>
-  </si>
-  <si>
-    <t>3:15pm</t>
-  </si>
-  <si>
-    <t>Pitti Palace and the Boboli Gardens — The gardens are the reason to go; climb to the top for the view back over the city</t>
-  </si>
-  <si>
-    <t>Oltrarno artisan workshops — Via Maggio and Santo Spirito — gilders, leatherworkers, restorers still working street level</t>
-  </si>
-  <si>
-    <t>7:15pm</t>
-  </si>
-  <si>
-    <t>Ponte Vecchio, then up to Piazzale Michelangelo — Sunset is around 8:00pm. Taxi up, walk down.</t>
-  </si>
-  <si>
-    <t>Taxi up, ~10 min</t>
-  </si>
-  <si>
-    <t>Dinner — Borgo San Jacopo — Michelin-starred, on the river, with a handful of window tables. Ask for one.</t>
-  </si>
-  <si>
-    <t>Walk down, ~15 min</t>
-  </si>
-  <si>
-    <t>Sat, Aug 29</t>
-  </si>
-  <si>
-    <t>FLORENCE → TUSCANY — Il Castelfalfi</t>
-  </si>
-  <si>
-    <t>9:00am</t>
-  </si>
-  <si>
-    <t>Check out; collect the rental car — The agencies cluster on Borgo Ognissanti, ~10 min on foot and just outside the ZTL — so you never drive into the centro storico. Have the IDP and licence ready.</t>
-  </si>
-  <si>
-    <t>9:45am</t>
-  </si>
-  <si>
-    <t>Southwest out of the city — Florence → Certaldo is about 45 minutes</t>
-  </si>
-  <si>
-    <t>Self-drive</t>
-  </si>
-  <si>
-    <t>10:30am</t>
-  </si>
-  <si>
-    <t>Certaldo Alto, by funicular — Boccaccio's birthplace — a walled brick town, the funicular climbs from Piazza Boccaccio in under two minutes</t>
-  </si>
-  <si>
-    <t>Arrive Certaldo</t>
-  </si>
-  <si>
-    <t>Info -&gt;</t>
-  </si>
-  <si>
-    <t>11:15am</t>
-  </si>
-  <si>
-    <t>Casa Boccaccio — The Decameron's author was born here; the house is now a small, quiet museum</t>
-  </si>
-  <si>
-    <t>Lunch on Via Boccaccio — A terrace table in the upper town before the drive on</t>
-  </si>
-  <si>
-    <t>On to Castelfalfi — About twenty-five minutes further into the Val d'Elsa</t>
-  </si>
-  <si>
-    <t>Driver</t>
-  </si>
-  <si>
-    <t>Check in — Il Castelfalfi — A restored 14th-century hamlet on a 2,700-acre estate, its own castle at the centre</t>
-  </si>
-  <si>
-    <t>Book -&gt;</t>
-  </si>
-  <si>
-    <t>The hamlet on foot — The piazza, the castle walls, the little church — all restored, none of it roped off</t>
-  </si>
-  <si>
     <t>Aperitivo at Ecrù — The estate's cocktail bar</t>
   </si>
   <si>
@@ -640,9 +652,6 @@
     <t>The village and a second cellar — Small enough to see on foot between tastings</t>
   </si>
   <si>
-    <t>5:30pm</t>
-  </si>
-  <si>
     <t>Back to Castelfalfi — About forty minutes</t>
   </si>
   <si>
@@ -737,9 +746,6 @@
   </si>
   <si>
     <t>The Piazzetta and the Gardens of Augustus — Gelato on the terrace above Via Krupp</t>
-  </si>
-  <si>
-    <t>6:15pm</t>
   </si>
   <si>
     <t>Ferry back to Naples — Check the final sailing when you arrive — the last fast boats go early evening, and missing one means a night on the island</t>
@@ -2085,7 +2091,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F137"/>
+  <dimension ref="A1:F138"/>
   <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2497,16 +2503,16 @@
         <v>48</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="F24" t="s">
-        <v>48</v>
+        <v>76</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -2517,16 +2523,16 @@
         <v>48</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>77</v>
+        <v>107</v>
+      </c>
+      <c r="F25" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -2537,50 +2543,50 @@
         <v>48</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="F26" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F26" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" t="s">
+        <v>48</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="F27" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="10">
+    <row r="29" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="10">
         <v>4</v>
       </c>
-      <c r="B28" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="F28" s="14" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>48</v>
-      </c>
-      <c r="B29" t="s">
-        <v>48</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="D29" s="4" t="s">
+      <c r="B29" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="E29" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="F29" t="s">
-        <v>48</v>
+      <c r="C29" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="F29" s="14" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -2591,16 +2597,16 @@
         <v>48</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>117</v>
+        <v>76</v>
+      </c>
+      <c r="F30" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -2619,8 +2625,8 @@
       <c r="E31" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="F31" t="s">
-        <v>48</v>
+      <c r="F31" s="7" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -2631,16 +2637,16 @@
         <v>48</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="F32" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
+      </c>
+      <c r="F32" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -2651,16 +2657,16 @@
         <v>48</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="F33" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2671,13 +2677,13 @@
         <v>48</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="F34" t="s">
         <v>48</v>
@@ -2691,13 +2697,13 @@
         <v>48</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>84</v>
+        <v>131</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F35" t="s">
         <v>48</v>
@@ -2711,16 +2717,16 @@
         <v>48</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>130</v>
+        <v>84</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E36" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="F36" s="7" t="s">
-        <v>123</v>
+      <c r="F36" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -2731,16 +2737,16 @@
         <v>48</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>134</v>
+        <v>63</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>77</v>
+        <v>127</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -2751,47 +2757,47 @@
         <v>48</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>103</v>
+        <v>138</v>
       </c>
       <c r="F38" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>48</v>
+      </c>
+      <c r="B39" t="s">
+        <v>48</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="E39" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="F39" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="40" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="10">
+    <row r="41" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="10">
         <v>5</v>
       </c>
-      <c r="B40" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="C40" s="11" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>48</v>
-      </c>
-      <c r="B41" t="s">
-        <v>48</v>
-      </c>
-      <c r="C41" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="E41" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>77</v>
+      <c r="B41" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="C41" s="11" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2802,13 +2808,13 @@
         <v>48</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>112</v>
+        <v>143</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F42" s="7" t="s">
         <v>77</v>
@@ -2822,16 +2828,16 @@
         <v>48</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>143</v>
+        <v>116</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="F43" t="s">
-        <v>48</v>
+        <v>146</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2842,16 +2848,16 @@
         <v>48</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>77</v>
+        <v>130</v>
+      </c>
+      <c r="F44" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -2862,16 +2868,16 @@
         <v>48</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -2882,16 +2888,16 @@
         <v>48</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>126</v>
+        <v>154</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -2902,16 +2908,16 @@
         <v>48</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>84</v>
+        <v>155</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="F47" t="s">
-        <v>48</v>
+        <v>130</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2922,13 +2928,13 @@
         <v>48</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>154</v>
+        <v>84</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>156</v>
+        <v>88</v>
       </c>
       <c r="F48" t="s">
         <v>48</v>
@@ -2942,50 +2948,50 @@
         <v>48</v>
       </c>
       <c r="C49" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="E49" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="F49" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>48</v>
+      </c>
+      <c r="B50" t="s">
+        <v>48</v>
+      </c>
+      <c r="C50" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="D49" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="E49" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="F49" s="7" t="s">
+      <c r="D50" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="E50" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="F50" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="51" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="10">
+    <row r="52" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="10">
         <v>6</v>
       </c>
-      <c r="B51" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="C51" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="F51" s="14" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>48</v>
-      </c>
-      <c r="B52" t="s">
-        <v>48</v>
-      </c>
-      <c r="C52" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="E52" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="F52" t="s">
-        <v>48</v>
+      <c r="B52" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="C52" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="F52" s="14" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -2996,13 +3002,13 @@
         <v>48</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E53" s="13" t="s">
-        <v>165</v>
+        <v>138</v>
       </c>
       <c r="F53" t="s">
         <v>48</v>
@@ -3016,16 +3022,16 @@
         <v>48</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E54" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="F54" s="7" t="s">
         <v>169</v>
+      </c>
+      <c r="F54" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -3042,10 +3048,10 @@
         <v>171</v>
       </c>
       <c r="E55" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="F55" t="s">
-        <v>48</v>
+        <v>172</v>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -3056,10 +3062,10 @@
         <v>48</v>
       </c>
       <c r="C56" s="12" t="s">
-        <v>78</v>
+        <v>173</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E56" s="13" t="s">
         <v>88</v>
@@ -3076,13 +3082,13 @@
         <v>48</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E57" s="13" t="s">
-        <v>174</v>
+        <v>88</v>
       </c>
       <c r="F57" t="s">
         <v>48</v>
@@ -3096,16 +3102,16 @@
         <v>48</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E58" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="F58" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
+      </c>
+      <c r="F58" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -3116,16 +3122,16 @@
         <v>48</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E59" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="F59" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="F59" s="7" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -3136,13 +3142,13 @@
         <v>48</v>
       </c>
       <c r="C60" s="12" t="s">
-        <v>104</v>
+        <v>84</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E60" s="13" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F60" t="s">
         <v>48</v>
@@ -3156,10 +3162,10 @@
         <v>48</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>89</v>
+        <v>181</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E61" s="13" t="s">
         <v>63</v>
@@ -3168,35 +3174,35 @@
         <v>48</v>
       </c>
     </row>
-    <row r="63" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="10">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>48</v>
+      </c>
+      <c r="B62" t="s">
+        <v>48</v>
+      </c>
+      <c r="C62" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="E62" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="F62" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="10">
         <v>7</v>
       </c>
-      <c r="B63" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="C63" s="11" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>48</v>
-      </c>
-      <c r="B64" t="s">
-        <v>48</v>
-      </c>
-      <c r="C64" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="D64" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="E64" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="F64" t="s">
-        <v>48</v>
+      <c r="B64" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="C64" s="11" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -3207,13 +3213,13 @@
         <v>48</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>183</v>
+        <v>116</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E65" s="13" t="s">
-        <v>57</v>
+        <v>169</v>
       </c>
       <c r="F65" t="s">
         <v>48</v>
@@ -3227,13 +3233,13 @@
         <v>48</v>
       </c>
       <c r="C66" s="12" t="s">
-        <v>143</v>
+        <v>187</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E66" s="13" t="s">
-        <v>88</v>
+        <v>57</v>
       </c>
       <c r="F66" t="s">
         <v>48</v>
@@ -3247,10 +3253,10 @@
         <v>48</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>186</v>
+        <v>147</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E67" s="13" t="s">
         <v>88</v>
@@ -3267,10 +3273,10 @@
         <v>48</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>78</v>
+        <v>190</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="E68" s="13" t="s">
         <v>88</v>
@@ -3287,13 +3293,13 @@
         <v>48</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="E69" s="13" t="s">
-        <v>165</v>
+        <v>88</v>
       </c>
       <c r="F69" t="s">
         <v>48</v>
@@ -3307,13 +3313,13 @@
         <v>48</v>
       </c>
       <c r="C70" s="12" t="s">
-        <v>190</v>
+        <v>81</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E70" s="13" t="s">
-        <v>192</v>
+        <v>169</v>
       </c>
       <c r="F70" t="s">
         <v>48</v>
@@ -3327,13 +3333,13 @@
         <v>48</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>84</v>
+        <v>194</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E71" s="13" t="s">
-        <v>88</v>
+        <v>196</v>
       </c>
       <c r="F71" t="s">
         <v>48</v>
@@ -3347,13 +3353,13 @@
         <v>48</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>194</v>
+        <v>84</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E72" s="13" t="s">
-        <v>174</v>
+        <v>88</v>
       </c>
       <c r="F72" t="s">
         <v>48</v>
@@ -3367,47 +3373,47 @@
         <v>48</v>
       </c>
       <c r="C73" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="E73" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="F73" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>48</v>
+      </c>
+      <c r="B74" t="s">
+        <v>48</v>
+      </c>
+      <c r="C74" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="D73" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="E73" s="13" t="s">
+      <c r="D74" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="E74" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="F73" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="75" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="10">
+      <c r="F74" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="76" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="10">
         <v>8</v>
       </c>
-      <c r="B75" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="C75" s="11" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>48</v>
-      </c>
-      <c r="B76" t="s">
-        <v>48</v>
-      </c>
-      <c r="C76" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="D76" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="E76" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="F76" t="s">
-        <v>48</v>
+      <c r="B76" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="C76" s="11" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -3418,13 +3424,13 @@
         <v>48</v>
       </c>
       <c r="C77" s="12" t="s">
-        <v>200</v>
+        <v>165</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E77" s="13" t="s">
-        <v>165</v>
+        <v>63</v>
       </c>
       <c r="F77" t="s">
         <v>48</v>
@@ -3438,13 +3444,13 @@
         <v>48</v>
       </c>
       <c r="C78" s="12" t="s">
-        <v>186</v>
+        <v>204</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="E78" s="13" t="s">
-        <v>57</v>
+        <v>169</v>
       </c>
       <c r="F78" t="s">
         <v>48</v>
@@ -3458,13 +3464,13 @@
         <v>48</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>203</v>
+        <v>190</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>205</v>
+        <v>57</v>
       </c>
       <c r="F79" t="s">
         <v>48</v>
@@ -3478,13 +3484,13 @@
         <v>48</v>
       </c>
       <c r="C80" s="12" t="s">
-        <v>190</v>
+        <v>207</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E80" s="13" t="s">
-        <v>88</v>
+        <v>209</v>
       </c>
       <c r="F80" t="s">
         <v>48</v>
@@ -3498,13 +3504,13 @@
         <v>48</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>207</v>
+        <v>194</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E81" s="13" t="s">
-        <v>174</v>
+        <v>88</v>
       </c>
       <c r="F81" t="s">
         <v>48</v>
@@ -3518,13 +3524,13 @@
         <v>48</v>
       </c>
       <c r="C82" s="12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E82" s="13" t="s">
-        <v>63</v>
+        <v>177</v>
       </c>
       <c r="F82" t="s">
         <v>48</v>
@@ -3538,10 +3544,10 @@
         <v>48</v>
       </c>
       <c r="C83" s="12" t="s">
-        <v>89</v>
+        <v>181</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E83" s="13" t="s">
         <v>63</v>
@@ -3550,38 +3556,38 @@
         <v>48</v>
       </c>
     </row>
-    <row r="85" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="10">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>48</v>
+      </c>
+      <c r="B84" t="s">
+        <v>48</v>
+      </c>
+      <c r="C84" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="E84" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="F84" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="10">
         <v>9</v>
       </c>
-      <c r="B85" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="C85" s="11" t="s">
-        <v>212</v>
-      </c>
-      <c r="F85" s="14" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>48</v>
-      </c>
-      <c r="B86" t="s">
-        <v>48</v>
-      </c>
-      <c r="C86" s="12" t="s">
-        <v>213</v>
-      </c>
-      <c r="D86" s="4" t="s">
+      <c r="B86" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="E86" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="F86" t="s">
-        <v>48</v>
+      <c r="C86" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="F86" s="14" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -3592,13 +3598,13 @@
         <v>48</v>
       </c>
       <c r="C87" s="12" t="s">
-        <v>183</v>
+        <v>216</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E87" s="13" t="s">
-        <v>216</v>
+        <v>169</v>
       </c>
       <c r="F87" t="s">
         <v>48</v>
@@ -3612,13 +3618,13 @@
         <v>48</v>
       </c>
       <c r="C88" s="12" t="s">
-        <v>143</v>
+        <v>187</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E88" s="13" t="s">
-        <v>88</v>
+        <v>219</v>
       </c>
       <c r="F88" t="s">
         <v>48</v>
@@ -3632,16 +3638,16 @@
         <v>48</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>218</v>
+        <v>147</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E89" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="F89" s="7" t="s">
-        <v>117</v>
+        <v>88</v>
+      </c>
+      <c r="F89" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
@@ -3658,10 +3664,10 @@
         <v>222</v>
       </c>
       <c r="E90" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="F90" t="s">
-        <v>48</v>
+        <v>223</v>
+      </c>
+      <c r="F90" s="7" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
@@ -3672,16 +3678,16 @@
         <v>48</v>
       </c>
       <c r="C91" s="12" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E91" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="F91" s="7" t="s">
-        <v>123</v>
+        <v>57</v>
+      </c>
+      <c r="F91" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
@@ -3692,16 +3698,16 @@
         <v>48</v>
       </c>
       <c r="C92" s="12" t="s">
-        <v>194</v>
+        <v>226</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E92" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="F92" t="s">
-        <v>48</v>
+        <v>76</v>
+      </c>
+      <c r="F92" s="7" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -3712,47 +3718,47 @@
         <v>48</v>
       </c>
       <c r="C93" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="E93" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="F93" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>48</v>
+      </c>
+      <c r="B94" t="s">
+        <v>48</v>
+      </c>
+      <c r="C94" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="D93" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="E93" s="13" t="s">
+      <c r="D94" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="E94" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="F93" s="7" t="s">
+      <c r="F94" s="7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="95" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="10">
+    <row r="96" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="10">
         <v>10</v>
       </c>
-      <c r="B95" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="C95" s="11" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>48</v>
-      </c>
-      <c r="B96" t="s">
-        <v>48</v>
-      </c>
-      <c r="C96" s="12" t="s">
-        <v>213</v>
-      </c>
-      <c r="D96" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="E96" s="13" t="s">
+      <c r="B96" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="F96" t="s">
-        <v>48</v>
+      <c r="C96" s="11" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
@@ -3763,7 +3769,7 @@
         <v>48</v>
       </c>
       <c r="C97" s="12" t="s">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="D97" s="4" t="s">
         <v>232</v>
@@ -3771,8 +3777,8 @@
       <c r="E97" s="13" t="s">
         <v>233</v>
       </c>
-      <c r="F97" s="7" t="s">
-        <v>234</v>
+      <c r="F97" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -3783,7 +3789,7 @@
         <v>48</v>
       </c>
       <c r="C98" s="12" t="s">
-        <v>166</v>
+        <v>234</v>
       </c>
       <c r="D98" s="4" t="s">
         <v>235</v>
@@ -3791,8 +3797,8 @@
       <c r="E98" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="F98" t="s">
-        <v>48</v>
+      <c r="F98" s="7" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -3803,16 +3809,16 @@
         <v>48</v>
       </c>
       <c r="C99" s="12" t="s">
-        <v>78</v>
+        <v>170</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E99" s="13" t="s">
-        <v>238</v>
-      </c>
-      <c r="F99" s="7" t="s">
-        <v>71</v>
+        <v>239</v>
+      </c>
+      <c r="F99" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
@@ -3823,16 +3829,16 @@
         <v>48</v>
       </c>
       <c r="C100" s="12" t="s">
-        <v>190</v>
+        <v>78</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E100" s="13" t="s">
-        <v>60</v>
+        <v>241</v>
       </c>
       <c r="F100" s="7" t="s">
-        <v>169</v>
+        <v>71</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -3843,16 +3849,16 @@
         <v>48</v>
       </c>
       <c r="C101" s="12" t="s">
-        <v>240</v>
+        <v>194</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E101" s="13" t="s">
-        <v>233</v>
-      </c>
-      <c r="F101" t="s">
-        <v>48</v>
+        <v>60</v>
+      </c>
+      <c r="F101" s="7" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -3863,50 +3869,50 @@
         <v>48</v>
       </c>
       <c r="C102" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="E102" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="F102" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>48</v>
+      </c>
+      <c r="B103" t="s">
+        <v>48</v>
+      </c>
+      <c r="C103" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="D102" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="E102" s="13" t="s">
+      <c r="D103" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="E103" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="F102" s="7" t="s">
+      <c r="F103" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="104" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="10">
+    <row r="105" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="10">
         <v>11</v>
       </c>
-      <c r="B104" s="10" t="s">
-        <v>243</v>
-      </c>
-      <c r="C104" s="11" t="s">
-        <v>244</v>
-      </c>
-      <c r="F104" s="14" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>48</v>
-      </c>
-      <c r="B105" t="s">
-        <v>48</v>
-      </c>
-      <c r="C105" s="12" t="s">
-        <v>213</v>
-      </c>
-      <c r="D105" s="4" t="s">
+      <c r="B105" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="E105" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="F105" t="s">
-        <v>48</v>
+      <c r="C105" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="F105" s="14" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
@@ -3917,13 +3923,13 @@
         <v>48</v>
       </c>
       <c r="C106" s="12" t="s">
-        <v>112</v>
+        <v>216</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E106" s="13" t="s">
-        <v>88</v>
+        <v>138</v>
       </c>
       <c r="F106" t="s">
         <v>48</v>
@@ -3937,13 +3943,13 @@
         <v>48</v>
       </c>
       <c r="C107" s="12" t="s">
-        <v>143</v>
+        <v>116</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E107" s="13" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="F107" t="s">
         <v>48</v>
@@ -3957,13 +3963,13 @@
         <v>48</v>
       </c>
       <c r="C108" s="12" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E108" s="13" t="s">
-        <v>249</v>
+        <v>63</v>
       </c>
       <c r="F108" t="s">
         <v>48</v>
@@ -3977,16 +3983,16 @@
         <v>48</v>
       </c>
       <c r="C109" s="12" t="s">
-        <v>203</v>
+        <v>149</v>
       </c>
       <c r="D109" s="4" t="s">
         <v>250</v>
       </c>
       <c r="E109" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="F109" s="7" t="s">
-        <v>123</v>
+        <v>251</v>
+      </c>
+      <c r="F109" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
@@ -3997,16 +4003,16 @@
         <v>48</v>
       </c>
       <c r="C110" s="12" t="s">
-        <v>58</v>
+        <v>207</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E110" s="13" t="s">
-        <v>252</v>
-      </c>
-      <c r="F110" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="F110" s="7" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -4017,13 +4023,13 @@
         <v>48</v>
       </c>
       <c r="C111" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D111" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="D111" s="4" t="s">
+      <c r="E111" s="13" t="s">
         <v>254</v>
-      </c>
-      <c r="E111" s="13" t="s">
-        <v>63</v>
       </c>
       <c r="F111" t="s">
         <v>48</v>
@@ -4037,47 +4043,47 @@
         <v>48</v>
       </c>
       <c r="C112" s="12" t="s">
-        <v>107</v>
+        <v>255</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E112" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="F112" s="7" t="s">
+      <c r="F112" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>48</v>
+      </c>
+      <c r="B113" t="s">
+        <v>48</v>
+      </c>
+      <c r="C113" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D113" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="E113" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="F113" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="114" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="10">
+    <row r="115" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="10">
         <v>12</v>
       </c>
-      <c r="B114" s="10" t="s">
-        <v>256</v>
-      </c>
-      <c r="C114" s="11" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>48</v>
-      </c>
-      <c r="B115" t="s">
-        <v>48</v>
-      </c>
-      <c r="C115" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="D115" s="4" t="s">
+      <c r="B115" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="E115" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="F115" t="s">
-        <v>48</v>
+      <c r="C115" s="11" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
@@ -4088,16 +4094,16 @@
         <v>48</v>
       </c>
       <c r="C116" s="12" t="s">
-        <v>186</v>
+        <v>165</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E116" s="13" t="s">
-        <v>260</v>
-      </c>
-      <c r="F116" s="7" t="s">
-        <v>71</v>
+        <v>63</v>
+      </c>
+      <c r="F116" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
@@ -4108,7 +4114,7 @@
         <v>48</v>
       </c>
       <c r="C117" s="12" t="s">
-        <v>58</v>
+        <v>190</v>
       </c>
       <c r="D117" s="4" t="s">
         <v>261</v>
@@ -4116,8 +4122,8 @@
       <c r="E117" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="F117" t="s">
-        <v>48</v>
+      <c r="F117" s="7" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
@@ -4128,16 +4134,16 @@
         <v>48</v>
       </c>
       <c r="C118" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D118" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="D118" s="4" t="s">
+      <c r="E118" s="13" t="s">
         <v>264</v>
       </c>
-      <c r="E118" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="F118" s="7" t="s">
-        <v>77</v>
+      <c r="F118" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
@@ -4148,13 +4154,13 @@
         <v>48</v>
       </c>
       <c r="C119" s="12" t="s">
-        <v>194</v>
+        <v>265</v>
       </c>
       <c r="D119" s="4" t="s">
         <v>266</v>
       </c>
       <c r="E119" s="13" t="s">
-        <v>88</v>
+        <v>267</v>
       </c>
       <c r="F119" s="7" t="s">
         <v>77</v>
@@ -4168,16 +4174,16 @@
         <v>48</v>
       </c>
       <c r="C120" s="12" t="s">
-        <v>64</v>
+        <v>198</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E120" s="13" t="s">
-        <v>268</v>
+        <v>88</v>
       </c>
       <c r="F120" s="7" t="s">
-        <v>269</v>
+        <v>77</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
@@ -4188,50 +4194,50 @@
         <v>48</v>
       </c>
       <c r="C121" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D121" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="E121" s="13" t="s">
         <v>270</v>
       </c>
-      <c r="D121" s="4" t="s">
+      <c r="F121" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="E121" s="13" t="s">
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>48</v>
+      </c>
+      <c r="B122" t="s">
+        <v>48</v>
+      </c>
+      <c r="C122" s="12" t="s">
         <v>272</v>
       </c>
-      <c r="F121" s="7" t="s">
+      <c r="D122" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="E122" s="13" t="s">
+        <v>274</v>
+      </c>
+      <c r="F122" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="123" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A123" s="10">
+    <row r="124" ht="20" customHeight="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="10">
         <v>13</v>
       </c>
-      <c r="B123" s="10" t="s">
-        <v>273</v>
-      </c>
-      <c r="C123" s="11" t="s">
-        <v>274</v>
-      </c>
-      <c r="F123" s="14" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
-        <v>48</v>
-      </c>
-      <c r="B124" t="s">
-        <v>48</v>
-      </c>
-      <c r="C124" s="12" t="s">
-        <v>213</v>
-      </c>
-      <c r="D124" s="4" t="s">
+      <c r="B124" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="E124" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="F124" t="s">
-        <v>48</v>
+      <c r="C124" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="F124" s="14" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
@@ -4242,13 +4248,13 @@
         <v>48</v>
       </c>
       <c r="C125" s="12" t="s">
-        <v>112</v>
+        <v>216</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E125" s="13" t="s">
-        <v>277</v>
+        <v>63</v>
       </c>
       <c r="F125" t="s">
         <v>48</v>
@@ -4262,13 +4268,13 @@
         <v>48</v>
       </c>
       <c r="C126" s="12" t="s">
-        <v>143</v>
+        <v>116</v>
       </c>
       <c r="D126" s="4" t="s">
         <v>278</v>
       </c>
       <c r="E126" s="13" t="s">
-        <v>57</v>
+        <v>279</v>
       </c>
       <c r="F126" t="s">
         <v>48</v>
@@ -4282,16 +4288,16 @@
         <v>48</v>
       </c>
       <c r="C127" s="12" t="s">
-        <v>49</v>
+        <v>147</v>
       </c>
       <c r="D127" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E127" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="F127" s="7" t="s">
-        <v>117</v>
+        <v>57</v>
+      </c>
+      <c r="F127" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
@@ -4302,16 +4308,16 @@
         <v>48</v>
       </c>
       <c r="C128" s="12" t="s">
-        <v>78</v>
+        <v>49</v>
       </c>
       <c r="D128" s="4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E128" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="F128" t="s">
-        <v>48</v>
+        <v>223</v>
+      </c>
+      <c r="F128" s="7" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
@@ -4322,16 +4328,16 @@
         <v>48</v>
       </c>
       <c r="C129" s="12" t="s">
-        <v>203</v>
+        <v>78</v>
       </c>
       <c r="D129" s="4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E129" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="F129" s="7" t="s">
-        <v>123</v>
+        <v>76</v>
+      </c>
+      <c r="F129" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
@@ -4342,16 +4348,16 @@
         <v>48</v>
       </c>
       <c r="C130" s="12" t="s">
-        <v>81</v>
+        <v>207</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E130" s="13" t="s">
-        <v>230</v>
-      </c>
-      <c r="F130" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="F130" s="7" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
@@ -4362,13 +4368,13 @@
         <v>48</v>
       </c>
       <c r="C131" s="12" t="s">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="D131" s="4" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E131" s="13" t="s">
-        <v>63</v>
+        <v>233</v>
       </c>
       <c r="F131" t="s">
         <v>48</v>
@@ -4382,47 +4388,47 @@
         <v>48</v>
       </c>
       <c r="C132" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="D132" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="E132" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="F132" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>48</v>
+      </c>
+      <c r="B133" t="s">
+        <v>48</v>
+      </c>
+      <c r="C133" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="D132" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="E132" s="13" t="s">
+      <c r="D133" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="E133" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="F132" s="7" t="s">
+      <c r="F133" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="134" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A134" s="10">
+    <row r="135" ht="20" customHeight="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="10">
         <v>14</v>
       </c>
-      <c r="B134" s="10" t="s">
-        <v>285</v>
-      </c>
-      <c r="C134" s="11" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A135" t="s">
-        <v>48</v>
-      </c>
-      <c r="B135" t="s">
-        <v>48</v>
-      </c>
-      <c r="C135" s="12" t="s">
+      <c r="B135" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="D135" s="4" t="s">
+      <c r="C135" s="11" t="s">
         <v>288</v>
-      </c>
-      <c r="E135" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="F135" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
@@ -4439,7 +4445,7 @@
         <v>290</v>
       </c>
       <c r="E136" s="13" t="s">
-        <v>291</v>
+        <v>83</v>
       </c>
       <c r="F136" t="s">
         <v>48</v>
@@ -4453,15 +4459,35 @@
         <v>48</v>
       </c>
       <c r="C137" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="D137" s="4" t="s">
         <v>292</v>
       </c>
-      <c r="D137" s="4" t="s">
+      <c r="E137" s="13" t="s">
         <v>293</v>
       </c>
-      <c r="E137" s="13" t="s">
+      <c r="F137" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>48</v>
+      </c>
+      <c r="B138" t="s">
+        <v>48</v>
+      </c>
+      <c r="C138" s="12" t="s">
         <v>294</v>
       </c>
-      <c r="F137" t="s">
+      <c r="D138" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="E138" s="13" t="s">
+        <v>296</v>
+      </c>
+      <c r="F138" t="s">
         <v>48</v>
       </c>
     </row>
@@ -4476,38 +4502,38 @@
     <hyperlink ref="F18" r:id="rId7"/>
     <hyperlink ref="F21" r:id="rId8"/>
     <hyperlink ref="F22" r:id="rId9"/>
-    <hyperlink ref="F25" r:id="rId10"/>
-    <hyperlink ref="F26" r:id="rId11"/>
-    <hyperlink ref="F30" r:id="rId12"/>
-    <hyperlink ref="F32" r:id="rId13"/>
-    <hyperlink ref="F36" r:id="rId14"/>
-    <hyperlink ref="F37" r:id="rId15"/>
-    <hyperlink ref="F38" r:id="rId16"/>
-    <hyperlink ref="F41" r:id="rId17"/>
-    <hyperlink ref="F42" r:id="rId18"/>
-    <hyperlink ref="F44" r:id="rId19"/>
-    <hyperlink ref="F45" r:id="rId20"/>
-    <hyperlink ref="F46" r:id="rId21"/>
-    <hyperlink ref="F49" r:id="rId22"/>
-    <hyperlink ref="F54" r:id="rId23"/>
-    <hyperlink ref="F58" r:id="rId24"/>
-    <hyperlink ref="F89" r:id="rId25"/>
-    <hyperlink ref="F91" r:id="rId26"/>
-    <hyperlink ref="F93" r:id="rId27"/>
-    <hyperlink ref="F97" r:id="rId28"/>
-    <hyperlink ref="F99" r:id="rId29"/>
-    <hyperlink ref="F100" r:id="rId30"/>
-    <hyperlink ref="F102" r:id="rId31"/>
-    <hyperlink ref="F109" r:id="rId32"/>
-    <hyperlink ref="F112" r:id="rId33"/>
-    <hyperlink ref="F116" r:id="rId34"/>
-    <hyperlink ref="F118" r:id="rId35"/>
-    <hyperlink ref="F119" r:id="rId36"/>
-    <hyperlink ref="F120" r:id="rId37"/>
-    <hyperlink ref="F121" r:id="rId38"/>
-    <hyperlink ref="F127" r:id="rId39"/>
-    <hyperlink ref="F129" r:id="rId40"/>
-    <hyperlink ref="F132" r:id="rId41"/>
+    <hyperlink ref="F24" r:id="rId10"/>
+    <hyperlink ref="F27" r:id="rId11"/>
+    <hyperlink ref="F31" r:id="rId12"/>
+    <hyperlink ref="F33" r:id="rId13"/>
+    <hyperlink ref="F37" r:id="rId14"/>
+    <hyperlink ref="F38" r:id="rId15"/>
+    <hyperlink ref="F39" r:id="rId16"/>
+    <hyperlink ref="F42" r:id="rId17"/>
+    <hyperlink ref="F43" r:id="rId18"/>
+    <hyperlink ref="F45" r:id="rId19"/>
+    <hyperlink ref="F46" r:id="rId20"/>
+    <hyperlink ref="F47" r:id="rId21"/>
+    <hyperlink ref="F50" r:id="rId22"/>
+    <hyperlink ref="F55" r:id="rId23"/>
+    <hyperlink ref="F59" r:id="rId24"/>
+    <hyperlink ref="F90" r:id="rId25"/>
+    <hyperlink ref="F92" r:id="rId26"/>
+    <hyperlink ref="F94" r:id="rId27"/>
+    <hyperlink ref="F98" r:id="rId28"/>
+    <hyperlink ref="F100" r:id="rId29"/>
+    <hyperlink ref="F101" r:id="rId30"/>
+    <hyperlink ref="F103" r:id="rId31"/>
+    <hyperlink ref="F110" r:id="rId32"/>
+    <hyperlink ref="F113" r:id="rId33"/>
+    <hyperlink ref="F117" r:id="rId34"/>
+    <hyperlink ref="F119" r:id="rId35"/>
+    <hyperlink ref="F120" r:id="rId36"/>
+    <hyperlink ref="F121" r:id="rId37"/>
+    <hyperlink ref="F122" r:id="rId38"/>
+    <hyperlink ref="F128" r:id="rId39"/>
+    <hyperlink ref="F130" r:id="rId40"/>
+    <hyperlink ref="F133" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -4530,48 +4556,48 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C2" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D2" t="s">
         <v>46</v>
       </c>
       <c r="E2" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F2">
         <v>3</v>
@@ -4583,24 +4609,24 @@
         <v>1571.58</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B3" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C3" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D3" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="E3" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="F3">
         <v>2</v>
@@ -4612,24 +4638,24 @@
         <v>1470</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B4" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C4" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="D4" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="E4" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="F4">
         <v>3</v>
@@ -4641,24 +4667,24 @@
         <v>3764.98</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B5" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C5" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D5" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E5" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F5">
         <v>2</v>
@@ -4670,24 +4696,24 @@
         <v>1071</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B6" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C6" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="D6" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E6" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="F6">
         <v>2</v>
@@ -4699,24 +4725,24 @@
         <v>3000</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B7" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C7" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D7" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E7" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -4728,7 +4754,7 @@
         <v>1000</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="16" customFormat="1" x14ac:dyDescent="0.25">
@@ -4745,7 +4771,7 @@
         <v>48</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F8" s="16">
         <v>13</v>
@@ -4783,24 +4809,24 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B2" s="15">
         <v>11877.56</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -4811,51 +4837,51 @@
         <v>1775</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B4" s="15">
         <v>1900</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B5" s="15">
         <v>2400</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B6" s="15">
         <v>400</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B7" s="17">
         <v>18352.559999999998</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -4880,237 +4906,237 @@
         <v>41</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B2" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="D2" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B3" t="s">
+        <v>346</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="D3" t="s">
+        <v>348</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>344</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>345</v>
-      </c>
-      <c r="D3" t="s">
-        <v>346</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B4" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D4" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B5" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D5" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B6" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="D6" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B7" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D7" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B8" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D8" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B9" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="D9" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B10" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="D10" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B11" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="D11" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B12" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D12" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B13" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="D13" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B14" t="s">
         <v>83</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D14" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -5121,7 +5147,7 @@
         <v>48</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
   </sheetData>
@@ -5158,16 +5184,16 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="E1" s="9" t="s">
         <v>45</v>
@@ -5178,16 +5204,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -5195,16 +5221,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>393</v>
-      </c>
-      <c r="D3" s="20" t="s">
-        <v>394</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -5212,16 +5238,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -5229,16 +5255,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -5246,16 +5272,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -5263,16 +5289,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -5280,16 +5306,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -5297,16 +5323,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -5314,16 +5340,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -5331,16 +5357,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5348,16 +5374,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -5365,16 +5391,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -5382,16 +5408,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="C14" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="D14" s="21" t="s">
         <v>417</v>
       </c>
-      <c r="D14" s="21" t="s">
-        <v>415</v>
-      </c>
       <c r="E14" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -5399,16 +5425,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -5416,16 +5442,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -5433,7 +5459,7 @@
         <v>48</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -5441,10 +5467,10 @@
         <v>48</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -5452,10 +5478,10 @@
         <v>48</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -5497,158 +5523,158 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B2" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="C2" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="E2" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="F2" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B3" t="s">
+        <v>444</v>
+      </c>
+      <c r="C3" t="s">
+        <v>445</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="E3" t="s">
+        <v>447</v>
+      </c>
+      <c r="F3" t="s">
+        <v>441</v>
+      </c>
+      <c r="G3" s="7" t="s">
         <v>442</v>
       </c>
-      <c r="C3" t="s">
+      <c r="H3" s="7" t="s">
         <v>443</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>444</v>
-      </c>
-      <c r="E3" t="s">
-        <v>445</v>
-      </c>
-      <c r="F3" t="s">
-        <v>439</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>440</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B4" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C4" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="E4" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="F4" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="C5" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="E5" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="F5" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B6" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="C6" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="E6" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="F6" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5662,7 +5688,7 @@
         <v>48</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Swap Florence hotel to the confirmed Helvetia&Bristol booking
Replaces the planned/quoted Casa G. Firenze with the actual Booking.com
reservation: Helvetia&Bristol Firenze (Starhotels Collezione), Aug 27-29,
$1,486 total. Removes the now-done "book Casa G." checklist item and
renumbers, and updates the lodging budget total accordingly. Booking
confirmation number, PIN, and payment details are intentionally left
out of this file since it deploys to a public site.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/italy-2026/dist/Italy 2026 (revised).xlsx
+++ b/italy-2026/dist/Italy 2026 (revised).xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1003" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="999" uniqueCount="463">
   <si>
     <t>ITALY 2026 PLAN</t>
   </si>
@@ -64,7 +64,7 @@
     <t>Chain story</t>
   </si>
   <si>
-    <t>Hotel Trame (Rome, independent) → Casa G. Firenze (Florence, Michelin Guide) → Il Castelfalfi (Tuscany, TUI Blue Selection) → De Bonart (Naples, Hilton Curio) → Anantara Convento (Amalfi, Minor / GHA) → The St. Regis Rome (Marriott Bonvoy)</t>
+    <t>Hotel Trame (Rome, independent) → Helvetia&amp;Bristol Firenze (Florence, Starhotels Collezione) → Il Castelfalfi (Tuscany, TUI Blue Selection) → De Bonart (Naples, Hilton Curio) → Anantara Convento (Amalfi, Minor / GHA) → The St. Regis Rome (Marriott Bonvoy)</t>
   </si>
   <si>
     <t>HOW TO READ THIS WORKBOOK</t>
@@ -361,7 +361,7 @@
     <t>Thu, Aug 27</t>
   </si>
   <si>
-    <t>ROME → FLORENCE — Casa G. Firenze</t>
+    <t>ROME → FLORENCE — Helvetia&amp;Bristol Firenze</t>
   </si>
   <si>
     <t>TRAVEL DAY</t>
@@ -397,312 +397,312 @@
     <t>12:45pm</t>
   </si>
   <si>
-    <t>Drop bags at Casa G. Firenze — Via dei Rondinelli, between the Duomo and Santa Maria Novella. Rooms are ready from 3:00pm; they will hold luggage until then.</t>
+    <t>Drop bags at Helvetia&amp;Bristol Firenze — Via Dei Pescioni 2, off Via de' Tornabuoni, in Santa Maria Novella. Rooms are ready from 3:00pm; they will hold luggage until then.</t>
+  </si>
+  <si>
+    <t>1:15pm</t>
+  </si>
+  <si>
+    <t>Lunch at the Mercato Centrale — Five minutes north — the upstairs food hall, no booking, no ceremony</t>
+  </si>
+  <si>
+    <t>Walk, ~5 min</t>
+  </si>
+  <si>
+    <t>2:45pm</t>
+  </si>
+  <si>
+    <t>First orientation walk — The Duomo and Baptistery from the outside, then Piazza della Repubblica and down to the Arno. The ticketed interiors are all tomorrow — today is just getting your bearings.</t>
+  </si>
+  <si>
+    <t>Unpack and reset — The train bought you an afternoon the drive would have eaten</t>
+  </si>
+  <si>
+    <t>6:45pm</t>
+  </si>
+  <si>
+    <t>Aperitivo at the hotel bar — A Belle Époque room to ease into Florence — no need to go anywhere</t>
+  </si>
+  <si>
+    <t>8:00pm</t>
+  </si>
+  <si>
+    <t>OPERA — La Traviata at St. Mark's Anglican — Via Maggio, across Ponte Santa Trinita — booked for arrival evening, comfortably clear now the train lands you at midday.</t>
+  </si>
+  <si>
+    <t>Walk, ~10 min</t>
+  </si>
+  <si>
+    <t>9:45pm</t>
+  </si>
+  <si>
+    <t>Dinner — Trattoria Sostanza — Cash only. The butter chicken and the tortino. Alternative: Buca dell'Orafo.</t>
+  </si>
+  <si>
+    <t>Fri, Aug 28</t>
+  </si>
+  <si>
+    <t>FLORENCE — the full day</t>
+  </si>
+  <si>
+    <t>8:15am</t>
+  </si>
+  <si>
+    <t>Accademia — David at first entry — Forty-five minutes is genuinely enough. Go straight down the hall.</t>
+  </si>
+  <si>
+    <t>Duomo — climb Brunelleschi's dome — 463 steps, timed slot, and much better before the day heats up</t>
+  </si>
+  <si>
+    <t>Walk, ~6 min</t>
+  </si>
+  <si>
+    <t>11:00am</t>
+  </si>
+  <si>
+    <t>Coffee on Piazza della Signoria — The Loggia dei Lanzi is an open-air sculpture hall and it is free</t>
+  </si>
+  <si>
+    <t>11:30am</t>
+  </si>
+  <si>
+    <t>Uffizi, guided — Botticelli, Leonardo, the Caravaggio room. Roughly two hours with a guide.</t>
+  </si>
+  <si>
+    <t>Walk, ~3 min</t>
+  </si>
+  <si>
+    <t>1:45pm</t>
+  </si>
+  <si>
+    <t>Lunch in the Oltrarno — Il Santo Bevitore — Or Gucci Osteria if you want the splurge. Trattoria Mario is the third option if you'd rather eat near San Lorenzo.</t>
+  </si>
+  <si>
+    <t>Cross Ponte Santa Trinita, ~8 min</t>
+  </si>
+  <si>
+    <t>3:15pm</t>
+  </si>
+  <si>
+    <t>Pitti Palace and the Boboli Gardens — The gardens are the reason to go; climb to the top for the view back over the city</t>
+  </si>
+  <si>
+    <t>Oltrarno artisan workshops — Via Maggio and Santo Spirito — gilders, leatherworkers, restorers still working street level</t>
+  </si>
+  <si>
+    <t>7:15pm</t>
+  </si>
+  <si>
+    <t>Ponte Vecchio, then up to Piazzale Michelangelo — Sunset is around 8:00pm. Taxi up, walk down.</t>
+  </si>
+  <si>
+    <t>Taxi up, ~10 min</t>
+  </si>
+  <si>
+    <t>Dinner — Borgo San Jacopo — Michelin-starred, on the river, with a handful of window tables. Ask for one.</t>
+  </si>
+  <si>
+    <t>Walk down, ~15 min</t>
+  </si>
+  <si>
+    <t>Sat, Aug 29</t>
+  </si>
+  <si>
+    <t>FLORENCE → TUSCANY — Il Castelfalfi</t>
+  </si>
+  <si>
+    <t>9:00am</t>
+  </si>
+  <si>
+    <t>Check out; collect the rental car — The agencies cluster on Borgo Ognissanti, ~10 min on foot and just outside the ZTL — so you never drive into the centro storico. Have the IDP and licence ready.</t>
+  </si>
+  <si>
+    <t>9:45am</t>
+  </si>
+  <si>
+    <t>Southwest out of the city — Florence → Certaldo is about 45 minutes</t>
+  </si>
+  <si>
+    <t>Self-drive</t>
+  </si>
+  <si>
+    <t>10:30am</t>
+  </si>
+  <si>
+    <t>Certaldo Alto, by funicular — Boccaccio's birthplace — a walled brick town, the funicular climbs from Piazza Boccaccio in under two minutes</t>
+  </si>
+  <si>
+    <t>Arrive Certaldo</t>
+  </si>
+  <si>
+    <t>11:15am</t>
+  </si>
+  <si>
+    <t>Casa Boccaccio — The Decameron's author was born here; the house is now a small, quiet museum</t>
+  </si>
+  <si>
+    <t>Lunch on Via Boccaccio — A terrace table in the upper town before the drive on</t>
+  </si>
+  <si>
+    <t>On to Castelfalfi — About twenty-five minutes further into the Val d'Elsa</t>
+  </si>
+  <si>
+    <t>Driver</t>
+  </si>
+  <si>
+    <t>Check in — Il Castelfalfi — A restored 14th-century hamlet on a 2,700-acre estate, its own castle at the centre</t>
+  </si>
+  <si>
+    <t>Book -&gt;</t>
+  </si>
+  <si>
+    <t>The hamlet on foot — The piazza, the castle walls, the little church — all restored, none of it roped off</t>
+  </si>
+  <si>
+    <t>7:00pm</t>
+  </si>
+  <si>
+    <t>Aperitivo at Ecrù — The estate's cocktail bar</t>
+  </si>
+  <si>
+    <t>Dinner — La Via del Sale — The estate's fine-dining room; the vegetables and olive oil are grown on the property</t>
+  </si>
+  <si>
+    <t>Sun, Aug 30</t>
+  </si>
+  <si>
+    <t>TUSCANY — San Gimignano and Volterra</t>
+  </si>
+  <si>
+    <t>Driver to San Gimignano — About twenty-five minutes</t>
+  </si>
+  <si>
+    <t>10:00am</t>
+  </si>
+  <si>
+    <t>The towers of San Gimignano — Fourteen of the original seventy-two medieval towers still stand — best seen from Piazza della Cisterna</t>
+  </si>
+  <si>
+    <t>The Collegiata — Ghirlandaio and Gozzoli frescoes wall to wall in a church the size of a chapel</t>
+  </si>
+  <si>
+    <t>12:30pm</t>
+  </si>
+  <si>
+    <t>Gelato at Dondoli — A two-time world gelato champion, right on Piazza della Cisterna</t>
+  </si>
+  <si>
+    <t>Lunch + a Vernaccia tasting — San Gimignano's own DOCG white, crisp and mineral, made for a hot afternoon</t>
+  </si>
+  <si>
+    <t>Driver to Volterra — About forty-five minutes</t>
+  </si>
+  <si>
+    <t>3:30pm</t>
+  </si>
+  <si>
+    <t>Piazza dei Priori and the Roman theatre — Tuscany's most complete medieval civic square, plus a 1st-century BC theatre still being excavated</t>
+  </si>
+  <si>
+    <t>Arrive Volterra</t>
+  </si>
+  <si>
+    <t>Alabaster workshops — A carving tradition here since Etruscan times — several studios welcome walk-ins</t>
+  </si>
+  <si>
+    <t>6:30pm</t>
+  </si>
+  <si>
+    <t>Drive back to Castelfalfi — About fifty minutes</t>
+  </si>
+  <si>
+    <t>Dinner at the resort — Or a quieter table down in Montaione village</t>
+  </si>
+  <si>
+    <t>Mon, Aug 31</t>
+  </si>
+  <si>
+    <t>TUSCANY — Montespertoli wine day</t>
+  </si>
+  <si>
+    <t>The estate's 27-hole course, or the spa — Tuscany's largest golf course, or a morning at the newly renovated spa</t>
+  </si>
+  <si>
+    <t>12:00pm</t>
+  </si>
+  <si>
+    <t>Driver to Montespertoli — About forty minutes</t>
+  </si>
+  <si>
+    <t>A Chianti Montespertoli estate — The smallest Chianti DOCG sub-zone, carved out of the old Colli Fiorentini in 1997 — quieter than Chianti Classico proper</t>
+  </si>
+  <si>
+    <t>1:30pm</t>
+  </si>
+  <si>
+    <t>Lunch among the vines</t>
+  </si>
+  <si>
+    <t>At the estate</t>
+  </si>
+  <si>
+    <t>The village and a second cellar — Small enough to see on foot between tastings</t>
+  </si>
+  <si>
+    <t>Back to Castelfalfi — About forty minutes</t>
+  </si>
+  <si>
+    <t>The pool or the spa terrace at sunset</t>
+  </si>
+  <si>
+    <t>Dinner — Giglio Blu or La Via del Sale — Something casual, or a second night at the estate's fine-dining room</t>
+  </si>
+  <si>
+    <t>Tue, Sep 1</t>
+  </si>
+  <si>
+    <t>TUSCANY → NAPLES — return the car in Florence, then the train</t>
+  </si>
+  <si>
+    <t>8:30am</t>
+  </si>
+  <si>
+    <t>Check out; drive to Florence — Back the way you came — about ninety minutes, less traffic than the Friday-afternoon drive in</t>
+  </si>
+  <si>
+    <t>Drop off the rental car — Borgo Ognissanti, near Firenze S.M.N. — reservation #21586310US4 ends here</t>
+  </si>
+  <si>
+    <t>Rental desk</t>
+  </si>
+  <si>
+    <t>Coffee, then the platform — A buffer before the train — Frecciarossa 9413 doesn't wait</t>
+  </si>
+  <si>
+    <t>12:48pm</t>
+  </si>
+  <si>
+    <t>Frecciarossa 9413 to Naples — Firenze S.M.N. → Napoli Centrale, direct — 3h15. Super Economy fare, from €71.80.</t>
+  </si>
+  <si>
+    <t>Train</t>
+  </si>
+  <si>
+    <t>4:03pm</t>
+  </si>
+  <si>
+    <t>Arrive Napoli Centrale</t>
+  </si>
+  <si>
+    <t>4:30pm</t>
+  </si>
+  <si>
+    <t>Check in — De Bonart, Curio Collection — An art palazzo on Via Partenope in Chiaia, facing the bay</t>
   </si>
   <si>
     <t>Trip.com -&gt;</t>
   </si>
   <si>
-    <t>1:15pm</t>
-  </si>
-  <si>
-    <t>Lunch at the Mercato Centrale — Five minutes north — the upstairs food hall, no booking, no ceremony</t>
-  </si>
-  <si>
-    <t>Walk, ~5 min</t>
-  </si>
-  <si>
-    <t>2:45pm</t>
-  </si>
-  <si>
-    <t>First orientation walk — The Duomo and Baptistery from the outside, then Piazza della Repubblica and down to the Arno. The ticketed interiors are all tomorrow — today is just getting your bearings.</t>
-  </si>
-  <si>
-    <t>Unpack and reset — The train bought you an afternoon the drive would have eaten</t>
-  </si>
-  <si>
-    <t>6:45pm</t>
-  </si>
-  <si>
-    <t>Aperitivo on the secret patio — Casa G.'s courtyard bar</t>
-  </si>
-  <si>
-    <t>8:00pm</t>
-  </si>
-  <si>
-    <t>OPERA — La Traviata at St. Mark's Anglican — Via Maggio, across Ponte Santa Trinita — booked for arrival evening, comfortably clear now the train lands you at midday.</t>
-  </si>
-  <si>
-    <t>Walk, ~10 min</t>
-  </si>
-  <si>
-    <t>9:45pm</t>
-  </si>
-  <si>
-    <t>Dinner — Trattoria Sostanza — Cash only. The butter chicken and the tortino. Alternative: Buca dell'Orafo.</t>
-  </si>
-  <si>
-    <t>Fri, Aug 28</t>
-  </si>
-  <si>
-    <t>FLORENCE — the full day</t>
-  </si>
-  <si>
-    <t>8:15am</t>
-  </si>
-  <si>
-    <t>Accademia — David at first entry — Forty-five minutes is genuinely enough. Go straight down the hall.</t>
-  </si>
-  <si>
-    <t>Duomo — climb Brunelleschi's dome — 463 steps, timed slot, and much better before the day heats up</t>
-  </si>
-  <si>
-    <t>Walk, ~6 min</t>
-  </si>
-  <si>
-    <t>11:00am</t>
-  </si>
-  <si>
-    <t>Coffee on Piazza della Signoria — The Loggia dei Lanzi is an open-air sculpture hall and it is free</t>
-  </si>
-  <si>
-    <t>11:30am</t>
-  </si>
-  <si>
-    <t>Uffizi, guided — Botticelli, Leonardo, the Caravaggio room. Roughly two hours with a guide.</t>
-  </si>
-  <si>
-    <t>Walk, ~3 min</t>
-  </si>
-  <si>
-    <t>1:45pm</t>
-  </si>
-  <si>
-    <t>Lunch in the Oltrarno — Il Santo Bevitore — Or Gucci Osteria if you want the splurge. Trattoria Mario is the third option if you'd rather eat near San Lorenzo.</t>
-  </si>
-  <si>
-    <t>Cross Ponte Santa Trinita, ~8 min</t>
-  </si>
-  <si>
-    <t>3:15pm</t>
-  </si>
-  <si>
-    <t>Pitti Palace and the Boboli Gardens — The gardens are the reason to go; climb to the top for the view back over the city</t>
-  </si>
-  <si>
-    <t>Oltrarno artisan workshops — Via Maggio and Santo Spirito — gilders, leatherworkers, restorers still working street level</t>
-  </si>
-  <si>
-    <t>7:15pm</t>
-  </si>
-  <si>
-    <t>Ponte Vecchio, then up to Piazzale Michelangelo — Sunset is around 8:00pm. Taxi up, walk down.</t>
-  </si>
-  <si>
-    <t>Taxi up, ~10 min</t>
-  </si>
-  <si>
-    <t>Dinner — Borgo San Jacopo — Michelin-starred, on the river, with a handful of window tables. Ask for one.</t>
-  </si>
-  <si>
-    <t>Walk down, ~15 min</t>
-  </si>
-  <si>
-    <t>Sat, Aug 29</t>
-  </si>
-  <si>
-    <t>FLORENCE → TUSCANY — Il Castelfalfi</t>
-  </si>
-  <si>
-    <t>9:00am</t>
-  </si>
-  <si>
-    <t>Check out; collect the rental car — The agencies cluster on Borgo Ognissanti, ~10 min on foot and just outside the ZTL — so you never drive into the centro storico. Have the IDP and licence ready.</t>
-  </si>
-  <si>
-    <t>9:45am</t>
-  </si>
-  <si>
-    <t>Southwest out of the city — Florence → Certaldo is about 45 minutes</t>
-  </si>
-  <si>
-    <t>Self-drive</t>
-  </si>
-  <si>
-    <t>10:30am</t>
-  </si>
-  <si>
-    <t>Certaldo Alto, by funicular — Boccaccio's birthplace — a walled brick town, the funicular climbs from Piazza Boccaccio in under two minutes</t>
-  </si>
-  <si>
-    <t>Arrive Certaldo</t>
-  </si>
-  <si>
-    <t>11:15am</t>
-  </si>
-  <si>
-    <t>Casa Boccaccio — The Decameron's author was born here; the house is now a small, quiet museum</t>
-  </si>
-  <si>
-    <t>Lunch on Via Boccaccio — A terrace table in the upper town before the drive on</t>
-  </si>
-  <si>
-    <t>On to Castelfalfi — About twenty-five minutes further into the Val d'Elsa</t>
-  </si>
-  <si>
-    <t>Driver</t>
-  </si>
-  <si>
-    <t>Check in — Il Castelfalfi — A restored 14th-century hamlet on a 2,700-acre estate, its own castle at the centre</t>
-  </si>
-  <si>
-    <t>Book -&gt;</t>
-  </si>
-  <si>
-    <t>The hamlet on foot — The piazza, the castle walls, the little church — all restored, none of it roped off</t>
-  </si>
-  <si>
-    <t>7:00pm</t>
-  </si>
-  <si>
-    <t>Aperitivo at Ecrù — The estate's cocktail bar</t>
-  </si>
-  <si>
-    <t>Dinner — La Via del Sale — The estate's fine-dining room; the vegetables and olive oil are grown on the property</t>
-  </si>
-  <si>
-    <t>Sun, Aug 30</t>
-  </si>
-  <si>
-    <t>TUSCANY — San Gimignano and Volterra</t>
-  </si>
-  <si>
-    <t>Driver to San Gimignano — About twenty-five minutes</t>
-  </si>
-  <si>
-    <t>10:00am</t>
-  </si>
-  <si>
-    <t>The towers of San Gimignano — Fourteen of the original seventy-two medieval towers still stand — best seen from Piazza della Cisterna</t>
-  </si>
-  <si>
-    <t>The Collegiata — Ghirlandaio and Gozzoli frescoes wall to wall in a church the size of a chapel</t>
-  </si>
-  <si>
-    <t>12:30pm</t>
-  </si>
-  <si>
-    <t>Gelato at Dondoli — A two-time world gelato champion, right on Piazza della Cisterna</t>
-  </si>
-  <si>
-    <t>Lunch + a Vernaccia tasting — San Gimignano's own DOCG white, crisp and mineral, made for a hot afternoon</t>
-  </si>
-  <si>
-    <t>Driver to Volterra — About forty-five minutes</t>
-  </si>
-  <si>
-    <t>3:30pm</t>
-  </si>
-  <si>
-    <t>Piazza dei Priori and the Roman theatre — Tuscany's most complete medieval civic square, plus a 1st-century BC theatre still being excavated</t>
-  </si>
-  <si>
-    <t>Arrive Volterra</t>
-  </si>
-  <si>
-    <t>Alabaster workshops — A carving tradition here since Etruscan times — several studios welcome walk-ins</t>
-  </si>
-  <si>
-    <t>6:30pm</t>
-  </si>
-  <si>
-    <t>Drive back to Castelfalfi — About fifty minutes</t>
-  </si>
-  <si>
-    <t>Dinner at the resort — Or a quieter table down in Montaione village</t>
-  </si>
-  <si>
-    <t>Mon, Aug 31</t>
-  </si>
-  <si>
-    <t>TUSCANY — Montespertoli wine day</t>
-  </si>
-  <si>
-    <t>The estate's 27-hole course, or the spa — Tuscany's largest golf course, or a morning at the newly renovated spa</t>
-  </si>
-  <si>
-    <t>12:00pm</t>
-  </si>
-  <si>
-    <t>Driver to Montespertoli — About forty minutes</t>
-  </si>
-  <si>
-    <t>A Chianti Montespertoli estate — The smallest Chianti DOCG sub-zone, carved out of the old Colli Fiorentini in 1997 — quieter than Chianti Classico proper</t>
-  </si>
-  <si>
-    <t>1:30pm</t>
-  </si>
-  <si>
-    <t>Lunch among the vines</t>
-  </si>
-  <si>
-    <t>At the estate</t>
-  </si>
-  <si>
-    <t>The village and a second cellar — Small enough to see on foot between tastings</t>
-  </si>
-  <si>
-    <t>Back to Castelfalfi — About forty minutes</t>
-  </si>
-  <si>
-    <t>The pool or the spa terrace at sunset</t>
-  </si>
-  <si>
-    <t>Dinner — Giglio Blu or La Via del Sale — Something casual, or a second night at the estate's fine-dining room</t>
-  </si>
-  <si>
-    <t>Tue, Sep 1</t>
-  </si>
-  <si>
-    <t>TUSCANY → NAPLES — return the car in Florence, then the train</t>
-  </si>
-  <si>
-    <t>8:30am</t>
-  </si>
-  <si>
-    <t>Check out; drive to Florence — Back the way you came — about ninety minutes, less traffic than the Friday-afternoon drive in</t>
-  </si>
-  <si>
-    <t>Drop off the rental car — Borgo Ognissanti, near Firenze S.M.N. — reservation #21586310US4 ends here</t>
-  </si>
-  <si>
-    <t>Rental desk</t>
-  </si>
-  <si>
-    <t>Coffee, then the platform — A buffer before the train — Frecciarossa 9413 doesn't wait</t>
-  </si>
-  <si>
-    <t>12:48pm</t>
-  </si>
-  <si>
-    <t>Frecciarossa 9413 to Naples — Firenze S.M.N. → Napoli Centrale, direct — 3h15. Super Economy fare, from €71.80.</t>
-  </si>
-  <si>
-    <t>Train</t>
-  </si>
-  <si>
-    <t>4:03pm</t>
-  </si>
-  <si>
-    <t>Arrive Napoli Centrale</t>
-  </si>
-  <si>
-    <t>4:30pm</t>
-  </si>
-  <si>
-    <t>Check in — De Bonart, Curio Collection — An art palazzo on Via Partenope in Chiaia, facing the bay</t>
-  </si>
-  <si>
     <t>Rooftop aperitivo — Vesuvius on one side, the bay on the other</t>
   </si>
   <si>
@@ -949,10 +949,10 @@
     <t>Florence</t>
   </si>
   <si>
-    <t>Casa G. Firenze</t>
-  </si>
-  <si>
-    <t>Independent / Michelin Guide</t>
+    <t>Helvetia&amp;Bristol Firenze</t>
+  </si>
+  <si>
+    <t>Starhotels Collezione</t>
   </si>
   <si>
     <t>Tuscany</t>
@@ -1006,7 +1006,7 @@
     <t>Lodging</t>
   </si>
   <si>
-    <t>6 hotels, 13 nights. Trame ($1,571.58), Castelfalfi ($3,764.98) and De Bonart ($1,071, confirmed) are actual bookings; Convento is a quote, 2 nights rather than 3. The St. Regis is still an estimate.</t>
+    <t>6 hotels, 13 nights. Trame ($1,571.58), Helvetia&amp;Bristol ($1,486), Castelfalfi ($3,764.98) and De Bonart ($1,071) are confirmed bookings; Convento is a quote, 2 nights rather than 3. The St. Regis is still an estimate.</t>
   </si>
   <si>
     <t>Holding the old total pending a re-quote: the rental drops from 14 days to 3 (Florence Aug 29 → Florence Sep 1, both ends the same city now), but a one-way-turned-round-trip re-quote could move that either way. New costs: the FCO private transfer (~€70–90), two Frecciarossa fares, and private drivers for both Naples↔Amalfi legs. Rome and FCO parking are gone entirely.</t>
@@ -1189,31 +1189,25 @@
     <t>Urgency</t>
   </si>
   <si>
-    <t>Book Casa G. Firenze for Aug 27–29</t>
-  </si>
-  <si>
-    <t>Two nights in Florence, wedged between Rome and Tuscany — the tightest hotel window on the trip.</t>
+    <t>Reserve dinners at Il Castelfalfi — La Via del Sale, Aug 29 &amp; 31</t>
+  </si>
+  <si>
+    <t>The estate's fine-dining room. Worth booking ahead even though the room itself is already confirmed.</t>
+  </si>
+  <si>
+    <t>THIS WEEK</t>
+  </si>
+  <si>
+    <t>Open -&gt;</t>
+  </si>
+  <si>
+    <t>Rebook the rental car — Florence pickup and drop-off, not FCO</t>
+  </si>
+  <si>
+    <t>Reservation #21586310US4 is still FCO Aug 24 → FCO Sep 6. It needs to become Borgo Ognissanti, Florence, Aug 29 → Florence Sep 1: three days rather than fourteen, both ends in the same city. A different pickup/drop-off city usually carries a fee, so the €1,087.81 quote will not hold — re-quote before cancelling.</t>
   </si>
   <si>
     <t>DO NOW</t>
-  </si>
-  <si>
-    <t>Open -&gt;</t>
-  </si>
-  <si>
-    <t>Reserve dinners at Il Castelfalfi — La Via del Sale, Aug 29 &amp; 31</t>
-  </si>
-  <si>
-    <t>The estate's fine-dining room. Worth booking ahead even though the room itself is already confirmed.</t>
-  </si>
-  <si>
-    <t>THIS WEEK</t>
-  </si>
-  <si>
-    <t>Rebook the rental car — Florence pickup and drop-off, not FCO</t>
-  </si>
-  <si>
-    <t>Reservation #21586310US4 is still FCO Aug 24 → FCO Sep 6. It needs to become Borgo Ognissanti, Florence, Aug 29 → Florence Sep 1: three days rather than fourteen, both ends in the same city. A different pickup/drop-off city usually carries a fee, so the €1,087.81 quote will not hold — re-quote before cancelling.</t>
   </si>
   <si>
     <t>Book the FCO → Hotel Trame private driver</t>
@@ -1480,12 +1474,12 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF9E4529"/>
+      <color rgb="FF8A6D1F"/>
       <sz val="9"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF8A6D1F"/>
+      <color rgb="FF9E4529"/>
       <sz val="9"/>
     </font>
     <font>
@@ -2666,7 +2660,7 @@
         <v>57</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>127</v>
+        <v>104</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2677,13 +2671,13 @@
         <v>48</v>
       </c>
       <c r="C34" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D34" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="E34" s="13" t="s">
         <v>129</v>
-      </c>
-      <c r="E34" s="13" t="s">
-        <v>130</v>
       </c>
       <c r="F34" t="s">
         <v>48</v>
@@ -2697,10 +2691,10 @@
         <v>48</v>
       </c>
       <c r="C35" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D35" s="4" t="s">
         <v>131</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>132</v>
       </c>
       <c r="E35" s="13" t="s">
         <v>60</v>
@@ -2720,7 +2714,7 @@
         <v>84</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E36" s="13" t="s">
         <v>63</v>
@@ -2737,16 +2731,16 @@
         <v>48</v>
       </c>
       <c r="C37" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="D37" s="4" t="s">
         <v>134</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>135</v>
       </c>
       <c r="E37" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="F37" s="7" t="s">
-        <v>127</v>
+      <c r="F37" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -2757,13 +2751,13 @@
         <v>48</v>
       </c>
       <c r="C38" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D38" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="D38" s="4" t="s">
+      <c r="E38" s="13" t="s">
         <v>137</v>
-      </c>
-      <c r="E38" s="13" t="s">
-        <v>138</v>
       </c>
       <c r="F38" s="7" t="s">
         <v>77</v>
@@ -2777,10 +2771,10 @@
         <v>48</v>
       </c>
       <c r="C39" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="D39" s="4" t="s">
         <v>139</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>140</v>
       </c>
       <c r="E39" s="13" t="s">
         <v>112</v>
@@ -2794,10 +2788,10 @@
         <v>5</v>
       </c>
       <c r="B41" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="C41" s="11" t="s">
         <v>141</v>
-      </c>
-      <c r="C41" s="11" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2808,13 +2802,13 @@
         <v>48</v>
       </c>
       <c r="C42" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="D42" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="D42" s="4" t="s">
-        <v>144</v>
-      </c>
       <c r="E42" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F42" s="7" t="s">
         <v>77</v>
@@ -2831,10 +2825,10 @@
         <v>116</v>
       </c>
       <c r="D43" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="E43" s="13" t="s">
         <v>145</v>
-      </c>
-      <c r="E43" s="13" t="s">
-        <v>146</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>77</v>
@@ -2848,13 +2842,13 @@
         <v>48</v>
       </c>
       <c r="C44" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="D44" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="D44" s="4" t="s">
-        <v>148</v>
-      </c>
       <c r="E44" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F44" t="s">
         <v>48</v>
@@ -2868,13 +2862,13 @@
         <v>48</v>
       </c>
       <c r="C45" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="D45" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="D45" s="4" t="s">
+      <c r="E45" s="13" t="s">
         <v>150</v>
-      </c>
-      <c r="E45" s="13" t="s">
-        <v>151</v>
       </c>
       <c r="F45" s="7" t="s">
         <v>77</v>
@@ -2888,13 +2882,13 @@
         <v>48</v>
       </c>
       <c r="C46" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="D46" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="D46" s="4" t="s">
+      <c r="E46" s="13" t="s">
         <v>153</v>
-      </c>
-      <c r="E46" s="13" t="s">
-        <v>154</v>
       </c>
       <c r="F46" s="7" t="s">
         <v>71</v>
@@ -2908,13 +2902,13 @@
         <v>48</v>
       </c>
       <c r="C47" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="D47" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="D47" s="4" t="s">
-        <v>156</v>
-      </c>
       <c r="E47" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>77</v>
@@ -2931,7 +2925,7 @@
         <v>84</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E48" s="13" t="s">
         <v>88</v>
@@ -2948,13 +2942,13 @@
         <v>48</v>
       </c>
       <c r="C49" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="D49" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="D49" s="4" t="s">
+      <c r="E49" s="13" t="s">
         <v>159</v>
-      </c>
-      <c r="E49" s="13" t="s">
-        <v>160</v>
       </c>
       <c r="F49" t="s">
         <v>48</v>
@@ -2971,10 +2965,10 @@
         <v>89</v>
       </c>
       <c r="D50" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E50" s="13" t="s">
         <v>161</v>
-      </c>
-      <c r="E50" s="13" t="s">
-        <v>162</v>
       </c>
       <c r="F50" s="7" t="s">
         <v>71</v>
@@ -2985,10 +2979,10 @@
         <v>6</v>
       </c>
       <c r="B52" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="C52" s="11" t="s">
         <v>163</v>
-      </c>
-      <c r="C52" s="11" t="s">
-        <v>164</v>
       </c>
       <c r="F52" s="14" t="s">
         <v>115</v>
@@ -3002,13 +2996,13 @@
         <v>48</v>
       </c>
       <c r="C53" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="D53" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="D53" s="4" t="s">
-        <v>166</v>
-      </c>
       <c r="E53" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F53" t="s">
         <v>48</v>
@@ -3022,13 +3016,13 @@
         <v>48</v>
       </c>
       <c r="C54" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="D54" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="D54" s="4" t="s">
+      <c r="E54" s="13" t="s">
         <v>168</v>
-      </c>
-      <c r="E54" s="13" t="s">
-        <v>169</v>
       </c>
       <c r="F54" t="s">
         <v>48</v>
@@ -3042,13 +3036,13 @@
         <v>48</v>
       </c>
       <c r="C55" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="D55" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="D55" s="4" t="s">
+      <c r="E55" s="13" t="s">
         <v>171</v>
-      </c>
-      <c r="E55" s="13" t="s">
-        <v>172</v>
       </c>
       <c r="F55" s="7" t="s">
         <v>104</v>
@@ -3062,10 +3056,10 @@
         <v>48</v>
       </c>
       <c r="C56" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="D56" s="4" t="s">
         <v>173</v>
-      </c>
-      <c r="D56" s="4" t="s">
-        <v>174</v>
       </c>
       <c r="E56" s="13" t="s">
         <v>88</v>
@@ -3085,7 +3079,7 @@
         <v>78</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E57" s="13" t="s">
         <v>88</v>
@@ -3105,10 +3099,10 @@
         <v>81</v>
       </c>
       <c r="D58" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="E58" s="13" t="s">
         <v>176</v>
-      </c>
-      <c r="E58" s="13" t="s">
-        <v>177</v>
       </c>
       <c r="F58" t="s">
         <v>48</v>
@@ -3125,13 +3119,13 @@
         <v>58</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E59" s="13" t="s">
         <v>57</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -3145,7 +3139,7 @@
         <v>84</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E60" s="13" t="s">
         <v>60</v>
@@ -3162,10 +3156,10 @@
         <v>48</v>
       </c>
       <c r="C61" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D61" s="4" t="s">
         <v>181</v>
-      </c>
-      <c r="D61" s="4" t="s">
-        <v>182</v>
       </c>
       <c r="E61" s="13" t="s">
         <v>63</v>
@@ -3185,7 +3179,7 @@
         <v>89</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E62" s="13" t="s">
         <v>63</v>
@@ -3199,10 +3193,10 @@
         <v>7</v>
       </c>
       <c r="B64" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="C64" s="11" t="s">
         <v>184</v>
-      </c>
-      <c r="C64" s="11" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -3216,10 +3210,10 @@
         <v>116</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E65" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F65" t="s">
         <v>48</v>
@@ -3233,10 +3227,10 @@
         <v>48</v>
       </c>
       <c r="C66" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="D66" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="D66" s="4" t="s">
-        <v>188</v>
       </c>
       <c r="E66" s="13" t="s">
         <v>57</v>
@@ -3253,10 +3247,10 @@
         <v>48</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E67" s="13" t="s">
         <v>88</v>
@@ -3273,10 +3267,10 @@
         <v>48</v>
       </c>
       <c r="C68" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="D68" s="4" t="s">
         <v>190</v>
-      </c>
-      <c r="D68" s="4" t="s">
-        <v>191</v>
       </c>
       <c r="E68" s="13" t="s">
         <v>88</v>
@@ -3296,7 +3290,7 @@
         <v>78</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E69" s="13" t="s">
         <v>88</v>
@@ -3316,10 +3310,10 @@
         <v>81</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E70" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F70" t="s">
         <v>48</v>
@@ -3333,13 +3327,13 @@
         <v>48</v>
       </c>
       <c r="C71" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="D71" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="D71" s="4" t="s">
+      <c r="E71" s="13" t="s">
         <v>195</v>
-      </c>
-      <c r="E71" s="13" t="s">
-        <v>196</v>
       </c>
       <c r="F71" t="s">
         <v>48</v>
@@ -3356,7 +3350,7 @@
         <v>84</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E72" s="13" t="s">
         <v>88</v>
@@ -3373,13 +3367,13 @@
         <v>48</v>
       </c>
       <c r="C73" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="D73" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="D73" s="4" t="s">
-        <v>199</v>
-      </c>
       <c r="E73" s="13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F73" t="s">
         <v>48</v>
@@ -3396,7 +3390,7 @@
         <v>89</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E74" s="13" t="s">
         <v>63</v>
@@ -3410,10 +3404,10 @@
         <v>8</v>
       </c>
       <c r="B76" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C76" s="11" t="s">
         <v>201</v>
-      </c>
-      <c r="C76" s="11" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -3424,10 +3418,10 @@
         <v>48</v>
       </c>
       <c r="C77" s="12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E77" s="13" t="s">
         <v>63</v>
@@ -3444,13 +3438,13 @@
         <v>48</v>
       </c>
       <c r="C78" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="D78" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="D78" s="4" t="s">
-        <v>205</v>
-      </c>
       <c r="E78" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F78" t="s">
         <v>48</v>
@@ -3464,10 +3458,10 @@
         <v>48</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E79" s="13" t="s">
         <v>57</v>
@@ -3484,13 +3478,13 @@
         <v>48</v>
       </c>
       <c r="C80" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="D80" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="D80" s="4" t="s">
+      <c r="E80" s="13" t="s">
         <v>208</v>
-      </c>
-      <c r="E80" s="13" t="s">
-        <v>209</v>
       </c>
       <c r="F80" t="s">
         <v>48</v>
@@ -3504,10 +3498,10 @@
         <v>48</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E81" s="13" t="s">
         <v>88</v>
@@ -3527,10 +3521,10 @@
         <v>105</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E82" s="13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F82" t="s">
         <v>48</v>
@@ -3544,10 +3538,10 @@
         <v>48</v>
       </c>
       <c r="C83" s="12" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E83" s="13" t="s">
         <v>63</v>
@@ -3567,7 +3561,7 @@
         <v>89</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E84" s="13" t="s">
         <v>63</v>
@@ -3581,10 +3575,10 @@
         <v>9</v>
       </c>
       <c r="B86" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="C86" s="11" t="s">
         <v>214</v>
-      </c>
-      <c r="C86" s="11" t="s">
-        <v>215</v>
       </c>
       <c r="F86" s="14" t="s">
         <v>115</v>
@@ -3598,13 +3592,13 @@
         <v>48</v>
       </c>
       <c r="C87" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="D87" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="D87" s="4" t="s">
-        <v>217</v>
-      </c>
       <c r="E87" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F87" t="s">
         <v>48</v>
@@ -3618,13 +3612,13 @@
         <v>48</v>
       </c>
       <c r="C88" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D88" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="E88" s="13" t="s">
         <v>218</v>
-      </c>
-      <c r="E88" s="13" t="s">
-        <v>219</v>
       </c>
       <c r="F88" t="s">
         <v>48</v>
@@ -3638,10 +3632,10 @@
         <v>48</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E89" s="13" t="s">
         <v>88</v>
@@ -3658,13 +3652,13 @@
         <v>48</v>
       </c>
       <c r="C90" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="D90" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="D90" s="4" t="s">
+      <c r="E90" s="13" t="s">
         <v>222</v>
-      </c>
-      <c r="E90" s="13" t="s">
-        <v>223</v>
       </c>
       <c r="F90" s="7" t="s">
         <v>121</v>
@@ -3678,10 +3672,10 @@
         <v>48</v>
       </c>
       <c r="C91" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="D91" s="4" t="s">
         <v>224</v>
-      </c>
-      <c r="D91" s="4" t="s">
-        <v>225</v>
       </c>
       <c r="E91" s="13" t="s">
         <v>57</v>
@@ -3698,16 +3692,16 @@
         <v>48</v>
       </c>
       <c r="C92" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="D92" s="4" t="s">
         <v>226</v>
-      </c>
-      <c r="D92" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="E92" s="13" t="s">
         <v>76</v>
       </c>
       <c r="F92" s="7" t="s">
-        <v>127</v>
+        <v>227</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -3718,7 +3712,7 @@
         <v>48</v>
       </c>
       <c r="C93" s="12" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D93" s="4" t="s">
         <v>228</v>
@@ -3769,7 +3763,7 @@
         <v>48</v>
       </c>
       <c r="C97" s="12" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D97" s="4" t="s">
         <v>232</v>
@@ -3809,7 +3803,7 @@
         <v>48</v>
       </c>
       <c r="C99" s="12" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D99" s="4" t="s">
         <v>238</v>
@@ -3849,7 +3843,7 @@
         <v>48</v>
       </c>
       <c r="C101" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D101" s="4" t="s">
         <v>242</v>
@@ -3923,13 +3917,13 @@
         <v>48</v>
       </c>
       <c r="C106" s="12" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D106" s="4" t="s">
         <v>247</v>
       </c>
       <c r="E106" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F106" t="s">
         <v>48</v>
@@ -3963,7 +3957,7 @@
         <v>48</v>
       </c>
       <c r="C108" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D108" s="4" t="s">
         <v>249</v>
@@ -3983,7 +3977,7 @@
         <v>48</v>
       </c>
       <c r="C109" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D109" s="4" t="s">
         <v>250</v>
@@ -4003,7 +3997,7 @@
         <v>48</v>
       </c>
       <c r="C110" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D110" s="4" t="s">
         <v>252</v>
@@ -4012,7 +4006,7 @@
         <v>57</v>
       </c>
       <c r="F110" s="7" t="s">
-        <v>127</v>
+        <v>227</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -4094,7 +4088,7 @@
         <v>48</v>
       </c>
       <c r="C116" s="12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D116" s="4" t="s">
         <v>260</v>
@@ -4114,7 +4108,7 @@
         <v>48</v>
       </c>
       <c r="C117" s="12" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D117" s="4" t="s">
         <v>261</v>
@@ -4174,7 +4168,7 @@
         <v>48</v>
       </c>
       <c r="C120" s="12" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D120" s="4" t="s">
         <v>268</v>
@@ -4248,7 +4242,7 @@
         <v>48</v>
       </c>
       <c r="C125" s="12" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D125" s="4" t="s">
         <v>277</v>
@@ -4288,7 +4282,7 @@
         <v>48</v>
       </c>
       <c r="C127" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D127" s="4" t="s">
         <v>280</v>
@@ -4314,7 +4308,7 @@
         <v>281</v>
       </c>
       <c r="E128" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F128" s="7" t="s">
         <v>121</v>
@@ -4348,7 +4342,7 @@
         <v>48</v>
       </c>
       <c r="C130" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D130" s="4" t="s">
         <v>283</v>
@@ -4357,7 +4351,7 @@
         <v>57</v>
       </c>
       <c r="F130" s="7" t="s">
-        <v>127</v>
+        <v>227</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
@@ -4506,34 +4500,33 @@
     <hyperlink ref="F27" r:id="rId11"/>
     <hyperlink ref="F31" r:id="rId12"/>
     <hyperlink ref="F33" r:id="rId13"/>
-    <hyperlink ref="F37" r:id="rId14"/>
-    <hyperlink ref="F38" r:id="rId15"/>
-    <hyperlink ref="F39" r:id="rId16"/>
-    <hyperlink ref="F42" r:id="rId17"/>
-    <hyperlink ref="F43" r:id="rId18"/>
-    <hyperlink ref="F45" r:id="rId19"/>
-    <hyperlink ref="F46" r:id="rId20"/>
-    <hyperlink ref="F47" r:id="rId21"/>
-    <hyperlink ref="F50" r:id="rId22"/>
-    <hyperlink ref="F55" r:id="rId23"/>
-    <hyperlink ref="F59" r:id="rId24"/>
-    <hyperlink ref="F90" r:id="rId25"/>
-    <hyperlink ref="F92" r:id="rId26"/>
-    <hyperlink ref="F94" r:id="rId27"/>
-    <hyperlink ref="F98" r:id="rId28"/>
-    <hyperlink ref="F100" r:id="rId29"/>
-    <hyperlink ref="F101" r:id="rId30"/>
-    <hyperlink ref="F103" r:id="rId31"/>
-    <hyperlink ref="F110" r:id="rId32"/>
-    <hyperlink ref="F113" r:id="rId33"/>
-    <hyperlink ref="F117" r:id="rId34"/>
-    <hyperlink ref="F119" r:id="rId35"/>
-    <hyperlink ref="F120" r:id="rId36"/>
-    <hyperlink ref="F121" r:id="rId37"/>
-    <hyperlink ref="F122" r:id="rId38"/>
-    <hyperlink ref="F128" r:id="rId39"/>
-    <hyperlink ref="F130" r:id="rId40"/>
-    <hyperlink ref="F133" r:id="rId41"/>
+    <hyperlink ref="F38" r:id="rId14"/>
+    <hyperlink ref="F39" r:id="rId15"/>
+    <hyperlink ref="F42" r:id="rId16"/>
+    <hyperlink ref="F43" r:id="rId17"/>
+    <hyperlink ref="F45" r:id="rId18"/>
+    <hyperlink ref="F46" r:id="rId19"/>
+    <hyperlink ref="F47" r:id="rId20"/>
+    <hyperlink ref="F50" r:id="rId21"/>
+    <hyperlink ref="F55" r:id="rId22"/>
+    <hyperlink ref="F59" r:id="rId23"/>
+    <hyperlink ref="F90" r:id="rId24"/>
+    <hyperlink ref="F92" r:id="rId25"/>
+    <hyperlink ref="F94" r:id="rId26"/>
+    <hyperlink ref="F98" r:id="rId27"/>
+    <hyperlink ref="F100" r:id="rId28"/>
+    <hyperlink ref="F101" r:id="rId29"/>
+    <hyperlink ref="F103" r:id="rId30"/>
+    <hyperlink ref="F110" r:id="rId31"/>
+    <hyperlink ref="F113" r:id="rId32"/>
+    <hyperlink ref="F117" r:id="rId33"/>
+    <hyperlink ref="F119" r:id="rId34"/>
+    <hyperlink ref="F120" r:id="rId35"/>
+    <hyperlink ref="F121" r:id="rId36"/>
+    <hyperlink ref="F122" r:id="rId37"/>
+    <hyperlink ref="F128" r:id="rId38"/>
+    <hyperlink ref="F130" r:id="rId39"/>
+    <hyperlink ref="F133" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -4609,7 +4602,7 @@
         <v>1571.58</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>127</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -4626,19 +4619,19 @@
         <v>113</v>
       </c>
       <c r="E3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F3">
         <v>2</v>
       </c>
       <c r="G3" s="15">
-        <v>735</v>
+        <v>743</v>
       </c>
       <c r="H3" s="15">
-        <v>1470</v>
+        <v>1486</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>127</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -4652,10 +4645,10 @@
         <v>314</v>
       </c>
       <c r="D4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F4">
         <v>3</v>
@@ -4667,7 +4660,7 @@
         <v>3764.98</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>127</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -4681,7 +4674,7 @@
         <v>317</v>
       </c>
       <c r="D5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E5" t="s">
         <v>245</v>
@@ -4696,7 +4689,7 @@
         <v>1071</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>127</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -4725,7 +4718,7 @@
         <v>3000</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>127</v>
+        <v>227</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -4754,7 +4747,7 @@
         <v>1000</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>127</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="16" customFormat="1" x14ac:dyDescent="0.25">
@@ -4780,7 +4773,7 @@
         <v>48</v>
       </c>
       <c r="H8" s="17">
-        <v>11877.56</v>
+        <v>11893.56</v>
       </c>
     </row>
   </sheetData>
@@ -4823,7 +4816,7 @@
         <v>328</v>
       </c>
       <c r="B2" s="15">
-        <v>11877.56</v>
+        <v>11893.56</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>329</v>
@@ -4878,7 +4871,7 @@
         <v>324</v>
       </c>
       <c r="B7" s="17">
-        <v>18352.559999999998</v>
+        <v>18368.559999999998</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>337</v>
@@ -4974,7 +4967,7 @@
         <v>349</v>
       </c>
       <c r="B5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C5" s="18" t="s">
         <v>353</v>
@@ -5110,7 +5103,7 @@
         <v>377</v>
       </c>
       <c r="B13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C13" s="18" t="s">
         <v>380</v>
@@ -5173,7 +5166,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="16" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -5243,8 +5236,8 @@
       <c r="C4" s="4" t="s">
         <v>398</v>
       </c>
-      <c r="D4" s="19" t="s">
-        <v>392</v>
+      <c r="D4" s="20" t="s">
+        <v>396</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>393</v>
@@ -5260,8 +5253,8 @@
       <c r="C5" s="4" t="s">
         <v>400</v>
       </c>
-      <c r="D5" s="19" t="s">
-        <v>392</v>
+      <c r="D5" s="20" t="s">
+        <v>396</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>393</v>
@@ -5294,8 +5287,8 @@
       <c r="C7" s="4" t="s">
         <v>404</v>
       </c>
-      <c r="D7" s="20" t="s">
-        <v>396</v>
+      <c r="D7" s="19" t="s">
+        <v>392</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>393</v>
@@ -5311,8 +5304,8 @@
       <c r="C8" s="4" t="s">
         <v>406</v>
       </c>
-      <c r="D8" s="20" t="s">
-        <v>396</v>
+      <c r="D8" s="19" t="s">
+        <v>392</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>393</v>
@@ -5328,8 +5321,8 @@
       <c r="C9" s="4" t="s">
         <v>408</v>
       </c>
-      <c r="D9" s="20" t="s">
-        <v>396</v>
+      <c r="D9" s="19" t="s">
+        <v>392</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>393</v>
@@ -5345,8 +5338,8 @@
       <c r="C10" s="4" t="s">
         <v>410</v>
       </c>
-      <c r="D10" s="20" t="s">
-        <v>396</v>
+      <c r="D10" s="19" t="s">
+        <v>392</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>393</v>
@@ -5362,8 +5355,8 @@
       <c r="C11" s="4" t="s">
         <v>412</v>
       </c>
-      <c r="D11" s="20" t="s">
-        <v>396</v>
+      <c r="D11" s="19" t="s">
+        <v>392</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>393</v>
@@ -5379,8 +5372,8 @@
       <c r="C12" s="4" t="s">
         <v>414</v>
       </c>
-      <c r="D12" s="20" t="s">
-        <v>396</v>
+      <c r="D12" s="21" t="s">
+        <v>415</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>393</v>
@@ -5391,13 +5384,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="D13" s="21" t="s">
         <v>415</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>417</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>393</v>
@@ -5414,7 +5407,7 @@
         <v>419</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>393</v>
@@ -5431,34 +5424,28 @@
         <v>421</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" s="6" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="22" t="s">
         <v>422</v>
       </c>
-      <c r="C16" s="4" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="23" t="s">
         <v>423</v>
       </c>
-      <c r="D16" s="21" t="s">
-        <v>417</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="22" t="s">
+      <c r="C18" s="2" t="s">
         <v>424</v>
       </c>
     </row>
@@ -5471,17 +5458,6 @@
       </c>
       <c r="C19" s="2" t="s">
         <v>426</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>48</v>
-      </c>
-      <c r="B20" s="23" t="s">
-        <v>427</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -5500,7 +5476,6 @@
     <hyperlink ref="E13" r:id="rId12"/>
     <hyperlink ref="E14" r:id="rId13"/>
     <hyperlink ref="E15" r:id="rId14"/>
-    <hyperlink ref="E16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -5523,28 +5498,28 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>428</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>429</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>430</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="E1" s="9" t="s">
         <v>431</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>432</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>433</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>434</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>435</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>436</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -5552,25 +5527,25 @@
         <v>306</v>
       </c>
       <c r="B2" t="s">
+        <v>435</v>
+      </c>
+      <c r="C2" t="s">
+        <v>436</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>437</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>438</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="F2" t="s">
         <v>439</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" s="7" t="s">
         <v>440</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" s="7" t="s">
         <v>441</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>442</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5578,51 +5553,51 @@
         <v>309</v>
       </c>
       <c r="B3" t="s">
+        <v>442</v>
+      </c>
+      <c r="C3" t="s">
+        <v>443</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>444</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>445</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>446</v>
-      </c>
-      <c r="E3" t="s">
-        <v>447</v>
-      </c>
       <c r="F3" t="s">
+        <v>439</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>440</v>
+      </c>
+      <c r="H3" s="7" t="s">
         <v>441</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>442</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>446</v>
+      </c>
+      <c r="B4" t="s">
+        <v>447</v>
+      </c>
+      <c r="C4" t="s">
         <v>448</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" s="4" t="s">
         <v>449</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>450</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="F4" t="s">
         <v>451</v>
       </c>
-      <c r="E4" t="s">
-        <v>452</v>
-      </c>
-      <c r="F4" t="s">
-        <v>453</v>
-      </c>
       <c r="G4" s="7" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5630,51 +5605,51 @@
         <v>318</v>
       </c>
       <c r="B5" t="s">
+        <v>452</v>
+      </c>
+      <c r="C5" t="s">
+        <v>453</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>454</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
         <v>455</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="F5" t="s">
         <v>456</v>
       </c>
-      <c r="E5" t="s">
-        <v>457</v>
-      </c>
-      <c r="F5" t="s">
-        <v>458</v>
-      </c>
       <c r="G5" s="7" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>457</v>
+      </c>
+      <c r="B6" t="s">
+        <v>458</v>
+      </c>
+      <c r="C6" t="s">
         <v>459</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" s="4" t="s">
         <v>460</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
         <v>461</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>462</v>
-      </c>
-      <c r="E6" t="s">
-        <v>463</v>
-      </c>
       <c r="F6" t="s">
+        <v>439</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>440</v>
+      </c>
+      <c r="H6" s="7" t="s">
         <v>441</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>442</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5688,7 +5663,7 @@
         <v>48</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cap every itinerary entry at three sentences
You asked for this after I argued the operational entries earned their length.
They did not — the facts survive the cut.

The two you named are the clearest cases. Vatican 539 → 374 characters, still
carrying the price, the entrance, the 30-minute voucher window, where the
Guided Tours desk is, the ID check, and that St Peter's is not included.
Borghese 425 → 283, keeping the meeting point, the purple shirt, the ID, the
headphones and the bag rule.

34 more rewrites across the rest. Nothing in the file now runs past three
sentences, details average 114 characters against 139 two commits ago, and no
time, price, address or booking constraint was dropped to get there.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/italy-2026/dist/Italy 2026 (revised).xlsx
+++ b/italy-2026/dist/Italy 2026 (revised).xlsx
@@ -178,7 +178,7 @@
     <t>12:35pm</t>
   </si>
   <si>
-    <t>Private driver to Hotel Trame — Pre-booked NCC, meeting you inside arrivals with a name board. Licensed cars may enter the ZTL, so you are dropped at the hotel door. On Uber: Italy has no UberX — the app offers only Uber Black, which costs more than a taxi. For a metered taxi use itTaxi or FreeNow, or a rank.</t>
+    <t>Private driver to Hotel Trame — Pre-booked NCC, meeting you inside arrivals with a name board; licensed cars may enter the ZTL, so you are dropped at the door. Italy has no UberX — the app offers only Uber Black, dearer than a taxi. Use itTaxi or FreeNow for a metered cab.</t>
   </si>
   <si>
     <t>Private transfer, ~45 min</t>
@@ -205,7 +205,7 @@
     <t>5:00pm</t>
   </si>
   <si>
-    <t>Shopping: Via del Corso up to the Spanish Steps — Timed on purpose: Aug 24 is a Monday, when Roman shops open late — most from 3:30 or 4pm until 7:30–8pm. Via del Corso is the chain high street, running from Piazza Venezia to Piazza del Popolo. Via dei Condotti at the top is the luxury row. Small independents may still be shut for the August break; the chains are not.</t>
+    <t>Shopping: Via del Corso up to the Spanish Steps — Aug 24 is a Monday, when Roman shops open late — most from 3:30 or 4pm until 7:30–8pm. Via del Corso is the chain high street, Piazza Venezia up to Piazza del Popolo; Via dei Condotti at the top is the luxury row. Small independents may still be shut for August, the chains not.</t>
   </si>
   <si>
     <t>Walk, ~10 min from Trevi</t>
@@ -235,7 +235,7 @@
     <t>8:00am</t>
   </si>
   <si>
-    <t>Vatican Gardens and Museums — arrive 8:00am, tour at 8:30am — Booked and paid, €90 for two. English, with earphones. Both names are on the ticket and ID is checked at the door, so carry it. Show the voucher to Customer Care outside the Viale Vaticano entrance 30 minutes before. After security, take the stairs at the far left of the entrance hall to the Guided Tours desk for tickets and coupons, then to the meeting point for earphones. Entrance is Passageway 2. Not changeable, not refundable. St Peter's is not included — ask your guide whether this tour uses the shortcut from the Sistine Chapel.</t>
+    <t>Vatican Gardens and Museums — arrive 8:00am, tour at 8:30am — Booked and paid, €90 for two: guided tour in English with earphones, entrance at Passageway 2. Show the voucher to Customer Care outside the Viale Vaticano entrance 30 minutes before, then collect tickets up the stairs at the far left of the hall, at the Guided Tours desk. Carry ID — both names are checked, it cannot be changed or refunded, and St Peter's is not included.</t>
   </si>
   <si>
     <t>Taxi, ~15 min</t>
@@ -301,7 +301,7 @@
     <t>8:45am</t>
   </si>
   <si>
-    <t>Baths of Caracalla — Go first, while it is quiet. Brick vaults at full height, huge bathing halls, patches of the original mosaic floor. Far emptier than anything else in ancient Rome at this hour.</t>
+    <t>Baths of Caracalla — Go first, while it is quiet — far emptier than anything else in ancient Rome at this hour. Brick vaults at full height, huge bathing halls, patches of the original mosaic floor.</t>
   </si>
   <si>
     <t>10:30am</t>
@@ -316,7 +316,7 @@
     <t>11:30am</t>
   </si>
   <si>
-    <t>Quick lunch in Monti — It has to be quick: the Borghese meeting point is a fifteen-minute taxi away and will not hold. Eat by 12:10 and you have a buffer. Roscioli had this slot but wants two unhurried hours — give it another lunch rather than rush it.</t>
+    <t>Quick lunch in Monti — Quick by necessity: the Borghese meeting point is a fifteen-minute taxi away and will not hold, so eat by 12:10. Roscioli had this slot but wants two unhurried hours. Give it another lunch rather than rush it.</t>
   </si>
   <si>
     <t>Walk, ~8 min</t>
@@ -325,7 +325,7 @@
     <t>12:45pm</t>
   </si>
   <si>
-    <t>Galleria Borghese — meet 12:45pm, entry at 1:00pm — Booked: skip-the-line entry for two, digital audioguide in English, two hours. Meet the host at the Fontana dei Mascheroni on Viale del Museo Borghese, in front of the gallery — purple Crown Tours shirt and a flag. Bring ID, your own headphones and a charged phone. No large bags inside; the cloakroom is free. Bernini's Apollo and Daphne and the Rape of Proserpina, plus six Caravaggios. You are let in and out on the clock.</t>
+    <t>Galleria Borghese — meet 12:45pm, entry at 1:00pm — Booked: skip-the-line entry for two, English audioguide, two hours on the clock. Meet the host at the Fontana dei Mascheroni in front of the gallery — purple Crown Tours shirt and a flag. Bring ID, your own headphones and a charged phone; no large bags inside, but the cloakroom is free.</t>
   </si>
   <si>
     <t>Gallery -&gt;</t>
@@ -391,7 +391,7 @@
     <t>12:10pm</t>
   </si>
   <si>
-    <t>Frecciarossa 9420 to Florence — Booked. Roma Termini 12:10 → Firenze S.M.N. 14:11, Executive, coach 1. Base fare, so it can be changed any number of times before departure.</t>
+    <t>Frecciarossa 9420 to Florence — Booked: Roma Termini 12:10 → Firenze S.M.N. 14:11, Executive, coach 1. Base fare, so it can be changed any number of times before departure.</t>
   </si>
   <si>
     <t>High-speed rail, 2h01</t>
@@ -409,7 +409,7 @@
     <t>2:25pm</t>
   </si>
   <si>
-    <t>Drop bags — The Hoxton — Via delle Mantellate 2, up by San Marco — 1.3km from the platform, so take a taxi with the bags. Rooms from 2:00pm; they will hold luggage until then. Checkout the 29th at noon. Room-only rate, so breakfast is on you both mornings.</t>
+    <t>Drop bags — The Hoxton — Via delle Mantellate 2, up by San Marco — 1.3km from the platform, so take a taxi with the bags. Rooms from 2:00pm, and they will hold luggage until then. Checkout the 29th at noon, room-only, so breakfast is on you.</t>
   </si>
   <si>
     <t>Taxi, ~8 min</t>
@@ -427,7 +427,7 @@
     <t>4:30pm</t>
   </si>
   <si>
-    <t>Climb Brunelleschi's dome — 4:30pm sharp — Booked: two Brunelleschi Passes, dome entry at the Porta della Mandorla. 463 steps, no lift. The slot cannot be changed and names are checked against ID, so be there by 4:15. The pass also covers the Bell Tower, Baptistery, museum and Santa Reparata crypt and runs through 29 August — which is why the museum sits on tomorrow.</t>
+    <t>Climb Brunelleschi's dome — 4:30pm sharp — Booked: two Brunelleschi Passes, dome entry at the Porta della Mandorla — 463 steps, no lift. The slot cannot be changed and names are checked against ID, so be there by 4:15. The pass also covers the Bell Tower, Baptistery, museum and crypt through 29 August.</t>
   </si>
   <si>
     <t>Duomo -&gt;</t>
@@ -460,7 +460,7 @@
     <t>8:15am</t>
   </si>
   <si>
-    <t>Pitti Palace and the Boboli Gardens — 8:15 is when the gates open, and that is the point — Boboli is terraced and unshaded, and unwalkable by mid-afternoon. The Palatine Gallery is hung floor to ceiling in the old manner. Climb to the top of the gardens for the view back over the city.</t>
+    <t>Pitti Palace and the Boboli Gardens — 8:15 is when the gates open, and that is the point — Boboli is terraced, unshaded and unwalkable by mid-afternoon. The Palatine Gallery is hung floor to ceiling in the old manner. Climb to the top of the gardens for the view back over the city.</t>
   </si>
   <si>
     <t>Coffee on the way down to Ponte Vecchio — Via de' Guicciardini runs from the palace gates to the bridge. Stop halfway.</t>
@@ -475,7 +475,7 @@
     <t>Cross Ponte Vecchio, ~6 min</t>
   </si>
   <si>
-    <t>Late lunch — 'Ino — Two hours from 12:15 puts you out at 2:30, which is when Oltrarno kitchens stop serving — so lunch is thirty seconds from the gallery door. Panini made to order, Tuscan wine by the glass, open through the afternoon. Il Santo Bevitore is the sit-down alternative if the tour runs short.</t>
+    <t>Late lunch — 'Ino — The Uffizi puts you out at 2:30, when Oltrarno kitchens stop serving, so lunch is thirty seconds from the gallery door. Panini made to order, Tuscan wine by the glass, open through the afternoon. Il Santo Bevitore is the sit-down alternative if the tour runs short.</t>
   </si>
   <si>
     <t>Walk, ~2 min</t>
@@ -484,13 +484,13 @@
     <t>4:00pm</t>
   </si>
   <si>
-    <t>Reverse Renaissance Walk — The centre backwards: Casa di Dante, then Orsanmichele, then Piazza della Signoria and the Loggia dei Lanzi — an open-air sculpture hall, free. Moved here from Thursday evening, which had no daylight for it.</t>
+    <t>Reverse Renaissance Walk — The centre backwards: Casa di Dante, Orsanmichele, then Piazza della Signoria and the Loggia dei Lanzi — an open-air sculpture hall, free.</t>
   </si>
   <si>
     <t>5:15pm</t>
   </si>
   <si>
-    <t>Opera del Duomo museum — Already paid — Thursday's Brunelleschi Pass runs to the 29th. Ghiberti's original Gates of Paradise and Michelangelo's late Pietà. Entrance is Piazza del Duomo 9.</t>
+    <t>Opera del Duomo museum — Already paid: Thursday's Brunelleschi Pass runs to the 29th. Ghiberti's original Gates of Paradise and Michelangelo's late Pietà, at Piazza del Duomo 9.</t>
   </si>
   <si>
     <t>6:30pm</t>
@@ -526,7 +526,7 @@
     <t>9:00am</t>
   </si>
   <si>
-    <t>Check out; collect the rental car — The agencies are on Borgo Ognissanti, just outside the ZTL, so you never drive into the centro storico. Twenty minutes downhill from the Hoxton — taxi with the luggage. Have the IDP and licence ready.</t>
+    <t>Check out; collect the rental car — The agencies are on Borgo Ognissanti, outside the ZTL, so you never drive into the centro storico. Twenty minutes downhill from the Hoxton, so taxi with the luggage. Have the IDP and licence ready.</t>
   </si>
   <si>
     <t>9:30am</t>
@@ -571,7 +571,7 @@
     <t>Self-drive</t>
   </si>
   <si>
-    <t>Check in — Il Castelfalfi — A restored 14th-century hamlet on a 2,700-acre estate, with its own castle. Deluxe Room with breakfast. Rooms from 3:00pm, checkout 11:00am on the 31st — which is why Monday starts at eight.</t>
+    <t>Check in — Il Castelfalfi — A restored 14th-century hamlet on a 2,700-acre estate, with its own castle. Deluxe Room with breakfast. Rooms from 3:00pm, checkout 11:00am on the 31st.</t>
   </si>
   <si>
     <t>Book -&gt;</t>
@@ -613,7 +613,7 @@
     <t>Gelato at Dondoli — A two-time world gelato champion on Piazza della Cisterna. Quick, before the horses</t>
   </si>
   <si>
-    <t>Horseback riding, lunch and a winery — San Gimignano Experience: about an hour in the saddle through vineyards, olive groves and woods, then a Tuscan lunch (antipasti, truffle lasagna, bread soup), a cellar tour and tastings of Chianti Classico, Vernaccia and Super Tuscans. No riding experience needed. Three to four hours; book ahead. Backup operator: CET Experience, cetexperience.it.</t>
+    <t>Horseback riding, lunch and a winery — An hour in the saddle through vineyards and olive groves, then a Tuscan lunch, a cellar tour and tastings of Chianti Classico, Vernaccia and Super Tuscans. No riding experience needed; three to four hours, and book ahead. Backup operator: CET Experience, cetexperience.it.</t>
   </si>
   <si>
     <t>Meet at the Bivio Volterra bus stop</t>
@@ -652,7 +652,7 @@
     <t>1:14pm</t>
   </si>
   <si>
-    <t>Frecciarossa 9587 to Naples — Booked. Firenze S.M.N. 13:14 → Napoli Centrale 16:23, direct via Rome, Executive, coach 1. The longest leg of the trip.</t>
+    <t>Frecciarossa 9587 to Naples — Booked: Firenze S.M.N. 13:14 → Napoli Centrale 16:23, direct via Rome, Executive, coach 1. The longest leg of the trip.</t>
   </si>
   <si>
     <t>High-speed rail, 3h09</t>
@@ -667,7 +667,7 @@
     <t>5:26pm</t>
   </si>
   <si>
-    <t>Campania Express to Sorrento — EAV 17:26 → Sorrento 18:35, direct. The tourist service, not the ordinary Circumvesuviana: reserved seats, air conditioning, room for a suitcase, €18pp. An hour's wait after the Frecciarossa, but it leaves from the same building — no crossing Naples with the bags.</t>
+    <t>Campania Express to Sorrento — EAV 17:26 → Sorrento 18:35, direct, €18pp. The tourist service, not the ordinary Circumvesuviana: reserved seats, air conditioning, room for a suitcase. An hour's wait after the Frecciarossa, but it leaves from the same building.</t>
   </si>
   <si>
     <t>Campania Express, 1h09</t>
@@ -685,7 +685,7 @@
     <t>6:50pm</t>
   </si>
   <si>
-    <t>Check in — Ara Maris Hotel &amp; Spa — Via Correale 15, a few minutes east of Piazza Tasso. Deluxe Sea View for the first four nights. Ask the desk to arrange the room move on the 4th while you are out at Amalfi.</t>
+    <t>Check in — Ara Maris Hotel &amp; Spa — Via Correale 15, a few minutes east of Piazza Tasso. Deluxe Sea View for the first four nights. Ask the desk to move the room on the 4th while you are out at Amalfi.</t>
   </si>
   <si>
     <t>7:15pm</t>
@@ -808,7 +808,7 @@
     <t>Ferry, ~35 min</t>
   </si>
   <si>
-    <t>Positano from the water, then from the stairs — The pastel town stacked straight up from Spiaggia Grande, and the majolica dome of Santa Maria Assunta. The best picture is from the boat coming in, so have the camera out before you dock.</t>
+    <t>Positano from the water, then from the stairs — The pastel town stacked straight up from Spiaggia Grande, under the majolica dome of Santa Maria Assunta. The best picture is from the boat coming in, so have the camera out before you dock.</t>
   </si>
   <si>
     <t>Lunch — Chez Black, on the beach — Right on Spiaggia Grande, and unpretentious despite the address. La Tagliata up in the hills is the alternative if you would rather climb.</t>
@@ -913,7 +913,7 @@
     <t>10:20am</t>
   </si>
   <si>
-    <t>Campania Express to Naples — Sorrento 10:20 → Napoli Piazza Garibaldi 11:34, direct, €18pp. Piazza Garibaldi is Napoli Centrale, so you step off one train where the next one leaves.</t>
+    <t>Campania Express to Naples — Sorrento 10:20 → Napoli Piazza Garibaldi 11:34, direct, €18pp. Piazza Garibaldi is Napoli Centrale, so you step off one train where the next leaves.</t>
   </si>
   <si>
     <t>Campania Express, 1h14</t>
@@ -928,7 +928,7 @@
     <t>11:55am</t>
   </si>
   <si>
-    <t>Pizza in Naples — the thing the replan took away — Bags into the station deposit, then the old city — Di Matteo and Sorbillo are both about twenty minutes up Via dei Tribunali. Naples came out of the itinerary altogether and this is the one window it gets back. If you would rather not risk it, there is good pizza in sight of the station.</t>
+    <t>Pizza in Naples — the thing the replan took away — Bags into the station deposit, then the old city — Di Matteo and Sorbillo are twenty minutes up Via dei Tribunali. Naples came out of the itinerary altogether, and this is the one window it gets back. If you would rather not risk it, there is good pizza in sight of the station.</t>
   </si>
   <si>
     <t>Walk, ~20 min</t>
@@ -958,7 +958,7 @@
     <t>3:20pm</t>
   </si>
   <si>
-    <t>Check in — Nomos Hotel — Via di San Paolo alla Regola, four minutes from Campo de' Fiori and two streets from where the trip began. Superior Double. Nothing is prepaid — you settle €530 with the hotel.</t>
+    <t>Check in — Nomos Hotel — Via di San Paolo alla Regola, four minutes from Campo de' Fiori and two streets from where the trip began. Superior Double, and nothing is prepaid — you settle €530 with the hotel.</t>
   </si>
   <si>
     <t>The Jewish Ghetto and the Portico d'Ottavia — Six minutes from the door, and the one corner of the centre you have not walked. Europe's oldest standing Jewish quarter, with the ruined portico built into the street</t>

</xml_diff>

<commit_message>
Ticketed stops carry directions only; prices and terms stay in Bookings
The booking rows already hold the price, the cancellation window, the operator
and the card that gets charged. Repeating them in the timeline meant the one
thing you actually need while standing outside Passageway 2 — which desk, which
stairs, what to bring — was buried in commercial detail you had already read.

So the eight ticketed stops now carry directions and nothing else. The Vatican
is the voucher, the desk, the stairs and the ID check. The Borghese is the
fountain, the purple shirt, and what to bring. The dome is the gate, the
deadline and the step count.

One fact had nowhere else to live: St Peter's is not part of the Vatican tour.
That moved up into the day-2 note rather than being dropped.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/italy-2026/dist/Italy 2026 (revised).xlsx
+++ b/italy-2026/dist/Italy 2026 (revised).xlsx
@@ -205,7 +205,7 @@
     <t>5:00pm</t>
   </si>
   <si>
-    <t>Shopping: Via del Corso up to the Spanish Steps — Aug 24 is a Monday, when Roman shops open late — most from 3:30 or 4pm until 7:30–8pm. Via del Corso is the chain high street, Piazza Venezia up to Piazza del Popolo; Via dei Condotti at the top is the luxury row. Small independents may still be shut for August, the chains not.</t>
+    <t>Shopping: Via del Corso up to the Spanish Steps — Via del Corso runs from Piazza Venezia to Piazza del Popolo; Via dei Condotti at the top is the luxury row. Monday hours, so shops open about 3:30–4pm and shut at 7:30–8pm. Small independents may still be closed for August.</t>
   </si>
   <si>
     <t>Walk, ~10 min from Trevi</t>
@@ -235,7 +235,7 @@
     <t>8:00am</t>
   </si>
   <si>
-    <t>Vatican Gardens and Museums — arrive 8:00am, tour at 8:30am — Booked and paid, €90 for two: guided tour in English with earphones, entrance at Passageway 2. Show the voucher to Customer Care outside the Viale Vaticano entrance 30 minutes before, then collect tickets up the stairs at the far left of the hall, at the Guided Tours desk. Carry ID — both names are checked, it cannot be changed or refunded, and St Peter's is not included.</t>
+    <t>Vatican Gardens and Museums — arrive 8:00am, tour at 8:30am — Show the voucher to Customer Care outside the Viale Vaticano entrance, 30 minutes before. After security, take the stairs at the far left of the hall to the Guided Tours desk for tickets, then on to the meeting point for earphones. Entrance is Passageway 2, and both names on the ticket are checked against ID.</t>
   </si>
   <si>
     <t>Taxi, ~15 min</t>
@@ -325,7 +325,7 @@
     <t>12:45pm</t>
   </si>
   <si>
-    <t>Galleria Borghese — meet 12:45pm, entry at 1:00pm — Booked: skip-the-line entry for two, English audioguide, two hours on the clock. Meet the host at the Fontana dei Mascheroni in front of the gallery — purple Crown Tours shirt and a flag. Bring ID, your own headphones and a charged phone; no large bags inside, but the cloakroom is free.</t>
+    <t>Galleria Borghese — meet 12:45pm, entry at 1:00pm — Meet the host at the Fontana dei Mascheroni, in front of the gallery — purple Crown Tours shirt and a flag. Bring ID, your own headphones and a charged phone. No large bags inside, but the cloakroom is free.</t>
   </si>
   <si>
     <t>Gallery -&gt;</t>
@@ -427,7 +427,7 @@
     <t>4:30pm</t>
   </si>
   <si>
-    <t>Climb Brunelleschi's dome — 4:30pm sharp — Booked: two Brunelleschi Passes, dome entry at the Porta della Mandorla — 463 steps, no lift. The slot cannot be changed and names are checked against ID, so be there by 4:15. The pass also covers the Bell Tower, Baptistery, museum and crypt through 29 August.</t>
+    <t>Climb Brunelleschi's dome — 4:30pm sharp — Entry is at the Porta della Mandorla — be there by 4:15 with ID, as the slot cannot be changed. 463 steps, no lift. The same pass covers the Bell Tower, Baptistery, museum and crypt through 29 August.</t>
   </si>
   <si>
     <t>Duomo -&gt;</t>
@@ -613,7 +613,7 @@
     <t>Gelato at Dondoli — A two-time world gelato champion on Piazza della Cisterna. Quick, before the horses</t>
   </si>
   <si>
-    <t>Horseback riding, lunch and a winery — An hour in the saddle through vineyards and olive groves, then a Tuscan lunch, a cellar tour and tastings of Chianti Classico, Vernaccia and Super Tuscans. No riding experience needed; three to four hours, and book ahead. Backup operator: CET Experience, cetexperience.it.</t>
+    <t>Horseback riding, lunch and a winery — Meets at the Bivio Volterra bus stop, 11am to 3pm. An hour in the saddle, then lunch, a cellar tour and tastings. No riding experience needed; backup operator is CET Experience, cetexperience.it.</t>
   </si>
   <si>
     <t>Meet at the Bivio Volterra bus stop</t>
@@ -667,7 +667,7 @@
     <t>5:26pm</t>
   </si>
   <si>
-    <t>Campania Express to Sorrento — EAV 17:26 → Sorrento 18:35, direct, €18pp. The tourist service, not the ordinary Circumvesuviana: reserved seats, air conditioning, room for a suitcase. An hour's wait after the Frecciarossa, but it leaves from the same building.</t>
+    <t>Campania Express to Sorrento — EAV 17:26 → Sorrento 18:35, direct. Platforms are downstairs from the Frecciarossa, signed EAV — no crossing Naples with the bags. Reserved seats, air conditioning and room for a suitcase.</t>
   </si>
   <si>
     <t>Campania Express, 1h09</t>
@@ -913,7 +913,7 @@
     <t>10:20am</t>
   </si>
   <si>
-    <t>Campania Express to Naples — Sorrento 10:20 → Napoli Piazza Garibaldi 11:34, direct, €18pp. Piazza Garibaldi is Napoli Centrale, so you step off one train where the next leaves.</t>
+    <t>Campania Express to Naples — Sorrento 10:20 → Napoli Piazza Garibaldi 11:34, direct. Piazza Garibaldi is Napoli Centrale, so you step off one train where the next leaves.</t>
   </si>
   <si>
     <t>Campania Express, 1h14</t>

</xml_diff>